<commit_message>
feat: equalize Top Videos & KOLs tables, support maximum rows display, real 5-platform scan progress modal, and 6-hour cloud cron
</commit_message>
<xml_diff>
--- a/exports/TikTok_Shop_US_Latest_Trends.xlsx
+++ b/exports/TikTok_Shop_US_Latest_Trends.xlsx
@@ -1410,7 +1410,7 @@
       </c>
       <c r="J21" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/STANLEY-Quencher-State-Tumbler-Quartz/dp/B0CP9Z56SW/ref=zg_bs_g_kitchen_d_sccl_2/134-3113057-6761362</t>
+          <t>https://www.amazon.com/STANLEY-Quencher-State-Tumbler-Quartz/dp/B0CP9Z56SW/ref=zg_bs_g_kitchen_d_sccl_2/134-1095087-0412057</t>
         </is>
       </c>
     </row>
@@ -1456,7 +1456,7 @@
       </c>
       <c r="J22" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/Medicube-Zero-Pore-Pads-Dual-Textured/dp/B09V7Z4TJG/ref=zg_bs_g_beauty_d_sccl_2/134-3113057-6761362</t>
+          <t>https://www.amazon.com/Medicube-Zero-Pore-Pads-Dual-Textured/dp/B09V7Z4TJG/ref=zg_bs_g_beauty_d_sccl_2/134-1095087-0412057</t>
         </is>
       </c>
     </row>
@@ -1502,7 +1502,7 @@
       </c>
       <c r="J23" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/HydroJug-Traveler-Resistant-Bottle-Reusable-Insulated/dp/B0CQVWT2NH/ref=zg_bs_g_kitchen_d_sccl_3/134-3113057-6761362</t>
+          <t>https://www.amazon.com/HydroJug-Traveler-Resistant-Bottle-Reusable-Insulated/dp/B0CQVWT2NH/ref=zg_bs_g_kitchen_d_sccl_3/134-1095087-0412057</t>
         </is>
       </c>
     </row>
@@ -1590,7 +1590,7 @@
       </c>
       <c r="J25" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/Apple-EarPods-Headphones-Built-Control/dp/B0DCH8VDXF/ref=zg_bs_g_electronics_d_sccl_2/134-3113057-6761362</t>
+          <t>https://www.amazon.com/Apple-EarPods-Headphones-Built-Control/dp/B0DCH8VDXF/ref=zg_bs_g_electronics_d_sccl_2/134-1095087-0412057</t>
         </is>
       </c>
     </row>
@@ -1636,7 +1636,7 @@
       </c>
       <c r="J26" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/Apple-AirTag-2nd-Generation-Precision/dp/B0GJTFXNRX/ref=zg_bs_g_electronics_d_sccl_3/134-3113057-6761362</t>
+          <t>https://www.amazon.com/Apple-AirTag-2nd-Generation-Precision/dp/B0GJTFXNRX/ref=zg_bs_g_electronics_d_sccl_3/134-1095087-0412057</t>
         </is>
       </c>
     </row>
@@ -1724,7 +1724,7 @@
       </c>
       <c r="J28" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/Apple-Cancellation-Translation-Headphones-High-Fidelity/dp/B0FQFB8FMG/ref=zg_bs_g_electronics_d_sccl_4/134-3113057-6761362</t>
+          <t>https://www.amazon.com/Apple-Cancellation-Translation-Headphones-High-Fidelity/dp/B0FQFB8FMG/ref=zg_bs_g_electronics_d_sccl_4/134-1095087-0412057</t>
         </is>
       </c>
     </row>
@@ -1770,7 +1770,7 @@
       </c>
       <c r="J29" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/Roku-Streaming-Stick-HD-2025/dp/B0DXXYS4BJ/ref=zg_bs_g_electronics_d_sccl_5/134-3113057-6761362</t>
+          <t>https://www.amazon.com/Roku-Streaming-Stick-HD-2025/dp/B0DXXYS4BJ/ref=zg_bs_g_electronics_d_sccl_5/134-1095087-0412057</t>
         </is>
       </c>
     </row>
@@ -1816,7 +1816,7 @@
       </c>
       <c r="J30" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/amazon-fire-tv-stick-4K-select/dp/B0C6W3D4RM/ref=zg_bs_g_electronics_d_sccl_6/134-3113057-6761362</t>
+          <t>https://www.amazon.com/amazon-fire-tv-stick-4K-select/dp/B0C6W3D4RM/ref=zg_bs_g_electronics_d_sccl_6/134-1095087-0412057</t>
         </is>
       </c>
     </row>
@@ -2128,19 +2128,19 @@
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>xrp price</t>
+          <t>dave franco</t>
         </is>
       </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
-          <t>Beauty &amp; Personal Care</t>
+          <t>Pet Supplies</t>
         </is>
       </c>
       <c r="D38" s="3" t="n">
         <v>78</v>
       </c>
       <c r="E38" s="3" t="n">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="F38" s="3" t="inlineStr">
         <is>
@@ -2154,17 +2154,17 @@
       </c>
       <c r="H38" s="4" t="inlineStr">
         <is>
-          <t>Đặt câu hỏi trúng nỗi đau thường ngày: 'Tại sao không ai nói cho tôi biết món đồ này sớm hơn?!'</t>
+          <t>Âm thanh bấm nút nhả cả búi lông chó rụng chỉ trong 1 giây: 'Mùa rụng lông không còn là ác mộng!'</t>
         </is>
       </c>
       <c r="I38" s="4" t="inlineStr">
         <is>
-          <t>Khách hàng mua sắm ngẫu hứng (Impulse Buyers) trên TikTok Shop US độ tuổi 18 - 45.</t>
+          <t>Hội những người 'nghiện' chó mèo (Dog/Cat Parents) tại US, chi tiêu mạnh tay cho thú cưng.</t>
         </is>
       </c>
       <c r="J38" s="5" t="inlineStr">
         <is>
-          <t>https://trends.google.com/trends/explore?geo=US&amp;q=xrp%20price</t>
+          <t>https://trends.google.com/trends/explore?geo=US&amp;q=dave%20franco</t>
         </is>
       </c>
     </row>
@@ -2174,7 +2174,7 @@
       </c>
       <c r="B39" s="4" t="inlineStr">
         <is>
-          <t>omaha weather</t>
+          <t>goog stock</t>
         </is>
       </c>
       <c r="C39" s="4" t="inlineStr">
@@ -2210,7 +2210,7 @@
       </c>
       <c r="J39" s="5" t="inlineStr">
         <is>
-          <t>https://trends.google.com/trends/explore?geo=US&amp;q=omaha%20weather</t>
+          <t>https://trends.google.com/trends/explore?geo=US&amp;q=goog%20stock</t>
         </is>
       </c>
     </row>
@@ -2220,7 +2220,7 @@
       </c>
       <c r="B40" s="4" t="inlineStr">
         <is>
-          <t>oil prices</t>
+          <t>aaron gordon</t>
         </is>
       </c>
       <c r="C40" s="4" t="inlineStr">
@@ -2246,17 +2246,17 @@
       </c>
       <c r="H40" s="4" t="inlineStr">
         <is>
-          <t>Before &amp; After cận cảnh lỗ chân lông: 'Dừng ngay nếu bạn vẫn đang nặn mụn hoặc dùng tẩy tế bào chết hạt to!'</t>
+          <t>Đặt câu hỏi trúng nỗi đau thường ngày: 'Tại sao không ai nói cho tôi biết món đồ này sớm hơn?!'</t>
         </is>
       </c>
       <c r="I40" s="4" t="inlineStr">
         <is>
-          <t>Gen Z &amp; Millennials (18-34 tuổi), Chăm sóc da mụn, tín đồ Skincare &amp; 'Clean Girl' aesthetic US.</t>
+          <t>Khách hàng mua sắm ngẫu hứng (Impulse Buyers) trên TikTok Shop US độ tuổi 18 - 45.</t>
         </is>
       </c>
       <c r="J40" s="5" t="inlineStr">
         <is>
-          <t>https://trends.google.com/trends/explore?geo=US&amp;q=oil%20prices</t>
+          <t>https://trends.google.com/trends/explore?geo=US&amp;q=aaron%20gordon</t>
         </is>
       </c>
     </row>
@@ -2266,12 +2266,12 @@
       </c>
       <c r="B41" s="4" t="inlineStr">
         <is>
-          <t>temperature</t>
+          <t>todd blanche joe digenova call</t>
         </is>
       </c>
       <c r="C41" s="4" t="inlineStr">
         <is>
-          <t>DIY, Craft &amp; POD</t>
+          <t>Gadgets &amp; Electronics</t>
         </is>
       </c>
       <c r="D41" s="3" t="n">
@@ -2292,17 +2292,17 @@
       </c>
       <c r="H41" s="4" t="inlineStr">
         <is>
-          <t>Quá trình máy khắc laser tên khách hàng lên gỗ/kim loại: 'Làm món quà độc nhất vô nhị tặng mẹ...'</t>
+          <t>Đặt câu hỏi trúng nỗi đau thường ngày: 'Tại sao không ai nói cho tôi biết món đồ này sớm hơn?!'</t>
         </is>
       </c>
       <c r="I41" s="4" t="inlineStr">
         <is>
-          <t>Người tìm quà tặng sinh nhật, kỷ niệm, Mother's Day, quà tân gia ý nghĩa quanh năm.</t>
+          <t>Khách hàng mua sắm ngẫu hứng (Impulse Buyers) trên TikTok Shop US độ tuổi 18 - 45.</t>
         </is>
       </c>
       <c r="J41" s="5" t="inlineStr">
         <is>
-          <t>https://trends.google.com/trends/explore?geo=US&amp;q=temperature</t>
+          <t>https://trends.google.com/trends/explore?geo=US&amp;q=todd%20blanche%20joe%20digenova%20call</t>
         </is>
       </c>
     </row>
@@ -2312,12 +2312,12 @@
       </c>
       <c r="B42" s="4" t="inlineStr">
         <is>
-          <t>clarity act</t>
+          <t>tropical storm weather forecast</t>
         </is>
       </c>
       <c r="C42" s="4" t="inlineStr">
         <is>
-          <t>DIY, Craft &amp; POD</t>
+          <t>Beauty &amp; Personal Care</t>
         </is>
       </c>
       <c r="D42" s="3" t="n">
@@ -2338,17 +2338,17 @@
       </c>
       <c r="H42" s="4" t="inlineStr">
         <is>
-          <t>Quá trình máy khắc laser tên khách hàng lên gỗ/kim loại: 'Làm món quà độc nhất vô nhị tặng mẹ...'</t>
+          <t>Đặt câu hỏi trúng nỗi đau thường ngày: 'Tại sao không ai nói cho tôi biết món đồ này sớm hơn?!'</t>
         </is>
       </c>
       <c r="I42" s="4" t="inlineStr">
         <is>
-          <t>Người tìm quà tặng sinh nhật, kỷ niệm, Mother's Day, quà tân gia ý nghĩa quanh năm.</t>
+          <t>Khách hàng mua sắm ngẫu hứng (Impulse Buyers) trên TikTok Shop US độ tuổi 18 - 45.</t>
         </is>
       </c>
       <c r="J42" s="5" t="inlineStr">
         <is>
-          <t>https://trends.google.com/trends/explore?geo=US&amp;q=clarity%20act</t>
+          <t>https://trends.google.com/trends/explore?geo=US&amp;q=tropical%20storm%20weather%20forecast</t>
         </is>
       </c>
     </row>
@@ -2358,7 +2358,7 @@
       </c>
       <c r="B43" s="4" t="inlineStr">
         <is>
-          <t>npr</t>
+          <t>nvda</t>
         </is>
       </c>
       <c r="C43" s="4" t="inlineStr">
@@ -2394,7 +2394,7 @@
       </c>
       <c r="J43" s="5" t="inlineStr">
         <is>
-          <t>https://trends.google.com/trends/explore?geo=US&amp;q=npr</t>
+          <t>https://trends.google.com/trends/explore?geo=US&amp;q=nvda</t>
         </is>
       </c>
     </row>
@@ -2404,7 +2404,7 @@
       </c>
       <c r="B44" s="4" t="inlineStr">
         <is>
-          <t>kaley cuoco</t>
+          <t>omaha weather</t>
         </is>
       </c>
       <c r="C44" s="4" t="inlineStr">
@@ -2440,7 +2440,7 @@
       </c>
       <c r="J44" s="5" t="inlineStr">
         <is>
-          <t>https://trends.google.com/trends/explore?geo=US&amp;q=kaley%20cuoco</t>
+          <t>https://trends.google.com/trends/explore?geo=US&amp;q=omaha%20weather</t>
         </is>
       </c>
     </row>
@@ -2450,12 +2450,12 @@
       </c>
       <c r="B45" s="4" t="inlineStr">
         <is>
-          <t>reba mcentire dolly parton emmy tribute</t>
+          <t>xrp price</t>
         </is>
       </c>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t>DIY, Craft &amp; POD</t>
+          <t>Beauty &amp; Personal Care</t>
         </is>
       </c>
       <c r="D45" s="3" t="n">
@@ -2476,17 +2476,17 @@
       </c>
       <c r="H45" s="4" t="inlineStr">
         <is>
-          <t>Quá trình máy khắc laser tên khách hàng lên gỗ/kim loại: 'Làm món quà độc nhất vô nhị tặng mẹ...'</t>
+          <t>Đặt câu hỏi trúng nỗi đau thường ngày: 'Tại sao không ai nói cho tôi biết món đồ này sớm hơn?!'</t>
         </is>
       </c>
       <c r="I45" s="4" t="inlineStr">
         <is>
-          <t>Người tìm quà tặng sinh nhật, kỷ niệm, Mother's Day, quà tân gia ý nghĩa quanh năm.</t>
+          <t>Khách hàng mua sắm ngẫu hứng (Impulse Buyers) trên TikTok Shop US độ tuổi 18 - 45.</t>
         </is>
       </c>
       <c r="J45" s="5" t="inlineStr">
         <is>
-          <t>https://trends.google.com/trends/explore?geo=US&amp;q=reba%20mcentire%20dolly%20parton%20emmy%20tribute</t>
+          <t>https://trends.google.com/trends/explore?geo=US&amp;q=xrp%20price</t>
         </is>
       </c>
     </row>
@@ -2496,7 +2496,7 @@
       </c>
       <c r="B46" s="4" t="inlineStr">
         <is>
-          <t>erin napier</t>
+          <t>clarity act</t>
         </is>
       </c>
       <c r="C46" s="4" t="inlineStr">
@@ -2532,7 +2532,7 @@
       </c>
       <c r="J46" s="5" t="inlineStr">
         <is>
-          <t>https://trends.google.com/trends/explore?geo=US&amp;q=erin%20napier</t>
+          <t>https://trends.google.com/trends/explore?geo=US&amp;q=clarity%20act</t>
         </is>
       </c>
     </row>
@@ -2542,12 +2542,12 @@
       </c>
       <c r="B47" s="4" t="inlineStr">
         <is>
-          <t>blake lively</t>
+          <t>temperature</t>
         </is>
       </c>
       <c r="C47" s="4" t="inlineStr">
         <is>
-          <t>Beauty &amp; Personal Care</t>
+          <t>DIY, Craft &amp; POD</t>
         </is>
       </c>
       <c r="D47" s="3" t="n">
@@ -2568,17 +2568,17 @@
       </c>
       <c r="H47" s="4" t="inlineStr">
         <is>
-          <t>Đặt câu hỏi trúng nỗi đau thường ngày: 'Tại sao không ai nói cho tôi biết món đồ này sớm hơn?!'</t>
+          <t>Quá trình máy khắc laser tên khách hàng lên gỗ/kim loại: 'Làm món quà độc nhất vô nhị tặng mẹ...'</t>
         </is>
       </c>
       <c r="I47" s="4" t="inlineStr">
         <is>
-          <t>Khách hàng mua sắm ngẫu hứng (Impulse Buyers) trên TikTok Shop US độ tuổi 18 - 45.</t>
+          <t>Người tìm quà tặng sinh nhật, kỷ niệm, Mother's Day, quà tân gia ý nghĩa quanh năm.</t>
         </is>
       </c>
       <c r="J47" s="5" t="inlineStr">
         <is>
-          <t>https://trends.google.com/trends/explore?geo=US&amp;q=blake%20lively</t>
+          <t>https://trends.google.com/trends/explore?geo=US&amp;q=temperature</t>
         </is>
       </c>
     </row>
@@ -5257,7 +5257,7 @@
       </c>
       <c r="I3" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/eos-Cashmere-Moisture-Lightweight-Non-Greasy/dp/B08KT2Z93D/ref=zg_bs_g_beauty_d_sccl_1/134-3113057-6761362</t>
+          <t>https://www.amazon.com/eos-Cashmere-Moisture-Lightweight-Non-Greasy/dp/B08KT2Z93D/ref=zg_bs_g_beauty_d_sccl_1/134-1095087-0412057</t>
         </is>
       </c>
     </row>
@@ -5298,7 +5298,7 @@
       </c>
       <c r="I4" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/Mighty-Patch-Hydrocolloid-Absorbing-count/dp/B074PVTPBW/ref=zg_bs_g_beauty_d_sccl_5/134-3113057-6761362</t>
+          <t>https://www.amazon.com/Mighty-Patch-Hydrocolloid-Absorbing-count/dp/B074PVTPBW/ref=zg_bs_g_beauty_d_sccl_5/134-1095087-0412057</t>
         </is>
       </c>
     </row>
@@ -5339,7 +5339,7 @@
       </c>
       <c r="I5" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/TERRO-T300-2-2-Pack-Liquid-Baits/dp/B00E4GACB8/ref=zg_bs_g_home-garden_d_sccl_1/134-3113057-6761362</t>
+          <t>https://www.amazon.com/TERRO-T300-2-2-Pack-Liquid-Baits/dp/B00E4GACB8/ref=zg_bs_g_home-garden_d_sccl_1/134-1095087-0412057</t>
         </is>
       </c>
     </row>
@@ -5380,7 +5380,7 @@
       </c>
       <c r="I6" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/Queen-Size-Piece-Sheet-Set/dp/B01M16WBW1/ref=zg_bs_g_home-garden_d_sccl_3/134-3113057-6761362</t>
+          <t>https://www.amazon.com/Queen-Size-Piece-Sheet-Set/dp/B01M16WBW1/ref=zg_bs_g_home-garden_d_sccl_3/134-1095087-0412057</t>
         </is>
       </c>
     </row>
@@ -5421,7 +5421,7 @@
       </c>
       <c r="I7" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/Dr-Elseys-Premium-Clumping-Litter/dp/B0009X29WK/ref=zg_bs_g_pet-supplies_d_sccl_1/134-3113057-6761362</t>
+          <t>https://www.amazon.com/Dr-Elseys-Premium-Clumping-Litter/dp/B0009X29WK/ref=zg_bs_g_pet-supplies_d_sccl_1/134-1095087-0412057</t>
         </is>
       </c>
     </row>
@@ -5462,7 +5462,7 @@
       </c>
       <c r="I8" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/Amazon-Basics-Leak-Proof-Quick-Dry-Absorbency/dp/B00MW8G62E/ref=zg_bs_g_pet-supplies_d_sccl_2/134-3113057-6761362</t>
+          <t>https://www.amazon.com/Amazon-Basics-Leak-Proof-Quick-Dry-Absorbency/dp/B00MW8G62E/ref=zg_bs_g_pet-supplies_d_sccl_2/134-1095087-0412057</t>
         </is>
       </c>
     </row>
@@ -5503,7 +5503,7 @@
       </c>
       <c r="I9" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/Purina-Fancy-Feast-Poultry-Collection/dp/B00JN9IWNG/ref=zg_bs_g_pet-supplies_d_sccl_3/134-3113057-6761362</t>
+          <t>https://www.amazon.com/Purina-Fancy-Feast-Poultry-Collection/dp/B00JN9IWNG/ref=zg_bs_g_pet-supplies_d_sccl_3/134-1095087-0412057</t>
         </is>
       </c>
     </row>
@@ -5544,7 +5544,7 @@
       </c>
       <c r="I10" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/Amazon-Basics-Cotton-Swabs-500ct/dp/B09541P9WH/ref=zg_bs_g_beauty_d_sccl_3/134-3113057-6761362</t>
+          <t>https://www.amazon.com/Amazon-Basics-Cotton-Swabs-500ct/dp/B09541P9WH/ref=zg_bs_g_beauty_d_sccl_3/134-1095087-0412057</t>
         </is>
       </c>
     </row>
@@ -5585,7 +5585,7 @@
       </c>
       <c r="I11" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/Clean-Skin-Club-Disposable-Sensitive/dp/B07PBXXNCY/ref=zg_bs_g_beauty_d_sccl_4/134-3113057-6761362</t>
+          <t>https://www.amazon.com/Clean-Skin-Club-Disposable-Sensitive/dp/B07PBXXNCY/ref=zg_bs_g_beauty_d_sccl_4/134-1095087-0412057</t>
         </is>
       </c>
     </row>
@@ -5626,7 +5626,7 @@
       </c>
       <c r="I12" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/Owala-FreeSip-Insulated-Stainless-BPA-Free/dp/B0BZYCJK89/ref=zg_bs_g_kitchen_d_sccl_1/134-3113057-6761362</t>
+          <t>https://www.amazon.com/Owala-FreeSip-Insulated-Stainless-BPA-Free/dp/B0BZYCJK89/ref=zg_bs_g_kitchen_d_sccl_1/134-1095087-0412057</t>
         </is>
       </c>
     </row>
@@ -5667,7 +5667,7 @@
       </c>
       <c r="I13" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/Owala-FreeSip-Insulated-Stainless-BPA-Free/dp/B0BZYCJK89/ref=zg_bs_g_home-garden_d_sccl_2/134-3113057-6761362</t>
+          <t>https://www.amazon.com/Owala-FreeSip-Insulated-Stainless-BPA-Free/dp/B0BZYCJK89/ref=zg_bs_g_home-garden_d_sccl_2/134-1095087-0412057</t>
         </is>
       </c>
     </row>
@@ -5708,7 +5708,7 @@
       </c>
       <c r="I14" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/Blink-Plus-Plan-monthly-auto-renewal/dp/B08JHCVHTY/ref=zg_bs_g_electronics_d_sccl_1/134-3113057-6761362</t>
+          <t>https://www.amazon.com/Blink-Plus-Plan-monthly-auto-renewal/dp/B08JHCVHTY/ref=zg_bs_g_electronics_d_sccl_1/134-1095087-0412057</t>
         </is>
       </c>
     </row>
@@ -5749,7 +5749,7 @@
       </c>
       <c r="I15" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/Owala-SmoothSip-Insulated-Stainless-Reusable/dp/B0DF3M7V3T/ref=zg_bs_g_kitchen_d_sccl_5/134-3113057-6761362</t>
+          <t>https://www.amazon.com/Owala-SmoothSip-Insulated-Stainless-Reusable/dp/B0DF3M7V3T/ref=zg_bs_g_kitchen_d_sccl_5/134-1095087-0412057</t>
         </is>
       </c>
     </row>
@@ -5790,7 +5790,7 @@
       </c>
       <c r="I16" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/Amazon-Basics-Cotton-Rounds-Count/dp/B09542G9ZN/ref=zg_bs_g_beauty_d_sccl_6/134-3113057-6761362</t>
+          <t>https://www.amazon.com/Amazon-Basics-Cotton-Rounds-Count/dp/B09542G9ZN/ref=zg_bs_g_beauty_d_sccl_6/134-1095087-0412057</t>
         </is>
       </c>
     </row>
@@ -5831,7 +5831,7 @@
       </c>
       <c r="I17" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/Etekcity-Multifunction-Stainless-Batteries-Included/dp/B0113UZJE2/ref=zg_bs_g_kitchen_d_sccl_4/134-3113057-6761362</t>
+          <t>https://www.amazon.com/Etekcity-Multifunction-Stainless-Batteries-Included/dp/B0113UZJE2/ref=zg_bs_g_kitchen_d_sccl_4/134-1095087-0412057</t>
         </is>
       </c>
     </row>
@@ -5872,7 +5872,7 @@
       </c>
       <c r="I18" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/Amazon-Basics-Microfiber-Lightweight-Wrinkle-free/dp/B0154ASID6/ref=zg_bs_g_home-garden_d_sccl_4/134-3113057-6761362</t>
+          <t>https://www.amazon.com/Amazon-Basics-Microfiber-Lightweight-Wrinkle-free/dp/B0154ASID6/ref=zg_bs_g_home-garden_d_sccl_4/134-1095087-0412057</t>
         </is>
       </c>
     </row>
@@ -5913,7 +5913,7 @@
       </c>
       <c r="I19" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/Electric-Flying-Insect-Trap-Starter/dp/B07T869RNY/ref=zg_bs_g_home-garden_d_sccl_6/134-3113057-6761362</t>
+          <t>https://www.amazon.com/Electric-Flying-Insect-Trap-Starter/dp/B07T869RNY/ref=zg_bs_g_home-garden_d_sccl_6/134-1095087-0412057</t>
         </is>
       </c>
     </row>
@@ -5954,7 +5954,7 @@
       </c>
       <c r="I20" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/Earth-Rated-Lavender-Scented-Completely/dp/B00BSYR7K8/ref=zg_bs_g_pet-supplies_d_sccl_5/134-3113057-6761362</t>
+          <t>https://www.amazon.com/Earth-Rated-Lavender-Scented-Completely/dp/B00BSYR7K8/ref=zg_bs_g_pet-supplies_d_sccl_5/134-1095087-0412057</t>
         </is>
       </c>
     </row>
@@ -5995,7 +5995,7 @@
       </c>
       <c r="I21" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/Toaster-Fits-anywhereTM-Kitchenware-Setting-Removable/dp/B0CYJBB2JQ/ref=zg_bs_g_kitchen_d_sccl_6/134-3113057-6761362</t>
+          <t>https://www.amazon.com/Toaster-Fits-anywhereTM-Kitchenware-Setting-Removable/dp/B0CYJBB2JQ/ref=zg_bs_g_kitchen_d_sccl_6/134-1095087-0412057</t>
         </is>
       </c>
     </row>
@@ -6036,7 +6036,7 @@
       </c>
       <c r="I22" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/ZEVO-Flying-Insect-Refills-Indoor/dp/B0C3FTCYZL/ref=zg_bs_g_home-garden_d_sccl_5/134-3113057-6761362</t>
+          <t>https://www.amazon.com/ZEVO-Flying-Insect-Refills-Indoor/dp/B0C3FTCYZL/ref=zg_bs_g_home-garden_d_sccl_5/134-1095087-0412057</t>
         </is>
       </c>
     </row>
@@ -6077,7 +6077,7 @@
       </c>
       <c r="I23" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/INABA-Grain-Free-Lickable-Squeezable-Vitamin/dp/B0B52D7BBD/ref=zg_bs_g_pet-supplies_d_sccl_4/134-3113057-6761362</t>
+          <t>https://www.amazon.com/INABA-Grain-Free-Lickable-Squeezable-Vitamin/dp/B0B52D7BBD/ref=zg_bs_g_pet-supplies_d_sccl_4/134-1095087-0412057</t>
         </is>
       </c>
     </row>
@@ -6118,7 +6118,7 @@
       </c>
       <c r="I24" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/Greenies-Pill-Pockets-Ingredients-Nutrients/dp/B008GRONV6/ref=zg_bs_g_pet-supplies_d_sccl_6/134-3113057-6761362</t>
+          <t>https://www.amazon.com/Greenies-Pill-Pockets-Ingredients-Nutrients/dp/B008GRONV6/ref=zg_bs_g_pet-supplies_d_sccl_6/134-1095087-0412057</t>
         </is>
       </c>
     </row>
@@ -7556,7 +7556,7 @@
       </c>
       <c r="L21" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/STANLEY-Quencher-State-Tumbler-Quartz/dp/B0CP9Z56SW/ref=zg_bs_g_kitchen_d_sccl_2/134-3113057-6761362</t>
+          <t>https://www.amazon.com/STANLEY-Quencher-State-Tumbler-Quartz/dp/B0CP9Z56SW/ref=zg_bs_g_kitchen_d_sccl_2/134-1095087-0412057</t>
         </is>
       </c>
     </row>
@@ -7610,7 +7610,7 @@
       </c>
       <c r="L22" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/Medicube-Zero-Pore-Pads-Dual-Textured/dp/B09V7Z4TJG/ref=zg_bs_g_beauty_d_sccl_2/134-3113057-6761362</t>
+          <t>https://www.amazon.com/Medicube-Zero-Pore-Pads-Dual-Textured/dp/B09V7Z4TJG/ref=zg_bs_g_beauty_d_sccl_2/134-1095087-0412057</t>
         </is>
       </c>
     </row>
@@ -7664,7 +7664,7 @@
       </c>
       <c r="L23" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/HydroJug-Traveler-Resistant-Bottle-Reusable-Insulated/dp/B0CQVWT2NH/ref=zg_bs_g_kitchen_d_sccl_3/134-3113057-6761362</t>
+          <t>https://www.amazon.com/HydroJug-Traveler-Resistant-Bottle-Reusable-Insulated/dp/B0CQVWT2NH/ref=zg_bs_g_kitchen_d_sccl_3/134-1095087-0412057</t>
         </is>
       </c>
     </row>
@@ -7768,7 +7768,7 @@
       </c>
       <c r="L25" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/eos-Cashmere-Moisture-Lightweight-Non-Greasy/dp/B08KT2Z93D/ref=zg_bs_g_beauty_d_sccl_1/134-3113057-6761362</t>
+          <t>https://www.amazon.com/eos-Cashmere-Moisture-Lightweight-Non-Greasy/dp/B08KT2Z93D/ref=zg_bs_g_beauty_d_sccl_1/134-1095087-0412057</t>
         </is>
       </c>
     </row>
@@ -7822,7 +7822,7 @@
       </c>
       <c r="L26" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/Mighty-Patch-Hydrocolloid-Absorbing-count/dp/B074PVTPBW/ref=zg_bs_g_beauty_d_sccl_5/134-3113057-6761362</t>
+          <t>https://www.amazon.com/Mighty-Patch-Hydrocolloid-Absorbing-count/dp/B074PVTPBW/ref=zg_bs_g_beauty_d_sccl_5/134-1095087-0412057</t>
         </is>
       </c>
     </row>
@@ -7876,7 +7876,7 @@
       </c>
       <c r="L27" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/TERRO-T300-2-2-Pack-Liquid-Baits/dp/B00E4GACB8/ref=zg_bs_g_home-garden_d_sccl_1/134-3113057-6761362</t>
+          <t>https://www.amazon.com/TERRO-T300-2-2-Pack-Liquid-Baits/dp/B00E4GACB8/ref=zg_bs_g_home-garden_d_sccl_1/134-1095087-0412057</t>
         </is>
       </c>
     </row>
@@ -7930,7 +7930,7 @@
       </c>
       <c r="L28" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/Queen-Size-Piece-Sheet-Set/dp/B01M16WBW1/ref=zg_bs_g_home-garden_d_sccl_3/134-3113057-6761362</t>
+          <t>https://www.amazon.com/Queen-Size-Piece-Sheet-Set/dp/B01M16WBW1/ref=zg_bs_g_home-garden_d_sccl_3/134-1095087-0412057</t>
         </is>
       </c>
     </row>
@@ -7984,7 +7984,7 @@
       </c>
       <c r="L29" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/Dr-Elseys-Premium-Clumping-Litter/dp/B0009X29WK/ref=zg_bs_g_pet-supplies_d_sccl_1/134-3113057-6761362</t>
+          <t>https://www.amazon.com/Dr-Elseys-Premium-Clumping-Litter/dp/B0009X29WK/ref=zg_bs_g_pet-supplies_d_sccl_1/134-1095087-0412057</t>
         </is>
       </c>
     </row>
@@ -8038,7 +8038,7 @@
       </c>
       <c r="L30" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/Amazon-Basics-Leak-Proof-Quick-Dry-Absorbency/dp/B00MW8G62E/ref=zg_bs_g_pet-supplies_d_sccl_2/134-3113057-6761362</t>
+          <t>https://www.amazon.com/Amazon-Basics-Leak-Proof-Quick-Dry-Absorbency/dp/B00MW8G62E/ref=zg_bs_g_pet-supplies_d_sccl_2/134-1095087-0412057</t>
         </is>
       </c>
     </row>
@@ -8092,7 +8092,7 @@
       </c>
       <c r="L31" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/Purina-Fancy-Feast-Poultry-Collection/dp/B00JN9IWNG/ref=zg_bs_g_pet-supplies_d_sccl_3/134-3113057-6761362</t>
+          <t>https://www.amazon.com/Purina-Fancy-Feast-Poultry-Collection/dp/B00JN9IWNG/ref=zg_bs_g_pet-supplies_d_sccl_3/134-1095087-0412057</t>
         </is>
       </c>
     </row>
@@ -8146,7 +8146,7 @@
       </c>
       <c r="L32" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/Amazon-Basics-Cotton-Swabs-500ct/dp/B09541P9WH/ref=zg_bs_g_beauty_d_sccl_3/134-3113057-6761362</t>
+          <t>https://www.amazon.com/Amazon-Basics-Cotton-Swabs-500ct/dp/B09541P9WH/ref=zg_bs_g_beauty_d_sccl_3/134-1095087-0412057</t>
         </is>
       </c>
     </row>
@@ -8200,7 +8200,7 @@
       </c>
       <c r="L33" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/Clean-Skin-Club-Disposable-Sensitive/dp/B07PBXXNCY/ref=zg_bs_g_beauty_d_sccl_4/134-3113057-6761362</t>
+          <t>https://www.amazon.com/Clean-Skin-Club-Disposable-Sensitive/dp/B07PBXXNCY/ref=zg_bs_g_beauty_d_sccl_4/134-1095087-0412057</t>
         </is>
       </c>
     </row>
@@ -8254,7 +8254,7 @@
       </c>
       <c r="L34" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/Owala-FreeSip-Insulated-Stainless-BPA-Free/dp/B0BZYCJK89/ref=zg_bs_g_kitchen_d_sccl_1/134-3113057-6761362</t>
+          <t>https://www.amazon.com/Owala-FreeSip-Insulated-Stainless-BPA-Free/dp/B0BZYCJK89/ref=zg_bs_g_kitchen_d_sccl_1/134-1095087-0412057</t>
         </is>
       </c>
     </row>
@@ -8308,7 +8308,7 @@
       </c>
       <c r="L35" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/Owala-FreeSip-Insulated-Stainless-BPA-Free/dp/B0BZYCJK89/ref=zg_bs_g_home-garden_d_sccl_2/134-3113057-6761362</t>
+          <t>https://www.amazon.com/Owala-FreeSip-Insulated-Stainless-BPA-Free/dp/B0BZYCJK89/ref=zg_bs_g_home-garden_d_sccl_2/134-1095087-0412057</t>
         </is>
       </c>
     </row>
@@ -8362,7 +8362,7 @@
       </c>
       <c r="L36" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/Blink-Plus-Plan-monthly-auto-renewal/dp/B08JHCVHTY/ref=zg_bs_g_electronics_d_sccl_1/134-3113057-6761362</t>
+          <t>https://www.amazon.com/Blink-Plus-Plan-monthly-auto-renewal/dp/B08JHCVHTY/ref=zg_bs_g_electronics_d_sccl_1/134-1095087-0412057</t>
         </is>
       </c>
     </row>
@@ -8416,7 +8416,7 @@
       </c>
       <c r="L37" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/Owala-SmoothSip-Insulated-Stainless-Reusable/dp/B0DF3M7V3T/ref=zg_bs_g_kitchen_d_sccl_5/134-3113057-6761362</t>
+          <t>https://www.amazon.com/Owala-SmoothSip-Insulated-Stainless-Reusable/dp/B0DF3M7V3T/ref=zg_bs_g_kitchen_d_sccl_5/134-1095087-0412057</t>
         </is>
       </c>
     </row>
@@ -8470,7 +8470,7 @@
       </c>
       <c r="L38" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/Apple-EarPods-Headphones-Built-Control/dp/B0DCH8VDXF/ref=zg_bs_g_electronics_d_sccl_2/134-3113057-6761362</t>
+          <t>https://www.amazon.com/Apple-EarPods-Headphones-Built-Control/dp/B0DCH8VDXF/ref=zg_bs_g_electronics_d_sccl_2/134-1095087-0412057</t>
         </is>
       </c>
     </row>
@@ -8524,7 +8524,7 @@
       </c>
       <c r="L39" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/Apple-AirTag-2nd-Generation-Precision/dp/B0GJTFXNRX/ref=zg_bs_g_electronics_d_sccl_3/134-3113057-6761362</t>
+          <t>https://www.amazon.com/Apple-AirTag-2nd-Generation-Precision/dp/B0GJTFXNRX/ref=zg_bs_g_electronics_d_sccl_3/134-1095087-0412057</t>
         </is>
       </c>
     </row>
@@ -8628,7 +8628,7 @@
       </c>
       <c r="L41" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/Amazon-Basics-Cotton-Rounds-Count/dp/B09542G9ZN/ref=zg_bs_g_beauty_d_sccl_6/134-3113057-6761362</t>
+          <t>https://www.amazon.com/Amazon-Basics-Cotton-Rounds-Count/dp/B09542G9ZN/ref=zg_bs_g_beauty_d_sccl_6/134-1095087-0412057</t>
         </is>
       </c>
     </row>
@@ -8682,7 +8682,7 @@
       </c>
       <c r="L42" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/Etekcity-Multifunction-Stainless-Batteries-Included/dp/B0113UZJE2/ref=zg_bs_g_kitchen_d_sccl_4/134-3113057-6761362</t>
+          <t>https://www.amazon.com/Etekcity-Multifunction-Stainless-Batteries-Included/dp/B0113UZJE2/ref=zg_bs_g_kitchen_d_sccl_4/134-1095087-0412057</t>
         </is>
       </c>
     </row>
@@ -8736,7 +8736,7 @@
       </c>
       <c r="L43" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/Amazon-Basics-Microfiber-Lightweight-Wrinkle-free/dp/B0154ASID6/ref=zg_bs_g_home-garden_d_sccl_4/134-3113057-6761362</t>
+          <t>https://www.amazon.com/Amazon-Basics-Microfiber-Lightweight-Wrinkle-free/dp/B0154ASID6/ref=zg_bs_g_home-garden_d_sccl_4/134-1095087-0412057</t>
         </is>
       </c>
     </row>
@@ -8790,7 +8790,7 @@
       </c>
       <c r="L44" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/Electric-Flying-Insect-Trap-Starter/dp/B07T869RNY/ref=zg_bs_g_home-garden_d_sccl_6/134-3113057-6761362</t>
+          <t>https://www.amazon.com/Electric-Flying-Insect-Trap-Starter/dp/B07T869RNY/ref=zg_bs_g_home-garden_d_sccl_6/134-1095087-0412057</t>
         </is>
       </c>
     </row>
@@ -8844,7 +8844,7 @@
       </c>
       <c r="L45" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/Earth-Rated-Lavender-Scented-Completely/dp/B00BSYR7K8/ref=zg_bs_g_pet-supplies_d_sccl_5/134-3113057-6761362</t>
+          <t>https://www.amazon.com/Earth-Rated-Lavender-Scented-Completely/dp/B00BSYR7K8/ref=zg_bs_g_pet-supplies_d_sccl_5/134-1095087-0412057</t>
         </is>
       </c>
     </row>
@@ -8898,7 +8898,7 @@
       </c>
       <c r="L46" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/Toaster-Fits-anywhereTM-Kitchenware-Setting-Removable/dp/B0CYJBB2JQ/ref=zg_bs_g_kitchen_d_sccl_6/134-3113057-6761362</t>
+          <t>https://www.amazon.com/Toaster-Fits-anywhereTM-Kitchenware-Setting-Removable/dp/B0CYJBB2JQ/ref=zg_bs_g_kitchen_d_sccl_6/134-1095087-0412057</t>
         </is>
       </c>
     </row>
@@ -8952,7 +8952,7 @@
       </c>
       <c r="L47" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/ZEVO-Flying-Insect-Refills-Indoor/dp/B0C3FTCYZL/ref=zg_bs_g_home-garden_d_sccl_5/134-3113057-6761362</t>
+          <t>https://www.amazon.com/ZEVO-Flying-Insect-Refills-Indoor/dp/B0C3FTCYZL/ref=zg_bs_g_home-garden_d_sccl_5/134-1095087-0412057</t>
         </is>
       </c>
     </row>
@@ -9006,7 +9006,7 @@
       </c>
       <c r="L48" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/INABA-Grain-Free-Lickable-Squeezable-Vitamin/dp/B0B52D7BBD/ref=zg_bs_g_pet-supplies_d_sccl_4/134-3113057-6761362</t>
+          <t>https://www.amazon.com/INABA-Grain-Free-Lickable-Squeezable-Vitamin/dp/B0B52D7BBD/ref=zg_bs_g_pet-supplies_d_sccl_4/134-1095087-0412057</t>
         </is>
       </c>
     </row>
@@ -9060,7 +9060,7 @@
       </c>
       <c r="L49" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/Greenies-Pill-Pockets-Ingredients-Nutrients/dp/B008GRONV6/ref=zg_bs_g_pet-supplies_d_sccl_6/134-3113057-6761362</t>
+          <t>https://www.amazon.com/Greenies-Pill-Pockets-Ingredients-Nutrients/dp/B008GRONV6/ref=zg_bs_g_pet-supplies_d_sccl_6/134-1095087-0412057</t>
         </is>
       </c>
     </row>
@@ -9114,7 +9114,7 @@
       </c>
       <c r="L50" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/Apple-Cancellation-Translation-Headphones-High-Fidelity/dp/B0FQFB8FMG/ref=zg_bs_g_electronics_d_sccl_4/134-3113057-6761362</t>
+          <t>https://www.amazon.com/Apple-Cancellation-Translation-Headphones-High-Fidelity/dp/B0FQFB8FMG/ref=zg_bs_g_electronics_d_sccl_4/134-1095087-0412057</t>
         </is>
       </c>
     </row>
@@ -9168,7 +9168,7 @@
       </c>
       <c r="L51" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/Roku-Streaming-Stick-HD-2025/dp/B0DXXYS4BJ/ref=zg_bs_g_electronics_d_sccl_5/134-3113057-6761362</t>
+          <t>https://www.amazon.com/Roku-Streaming-Stick-HD-2025/dp/B0DXXYS4BJ/ref=zg_bs_g_electronics_d_sccl_5/134-1095087-0412057</t>
         </is>
       </c>
     </row>
@@ -9222,7 +9222,7 @@
       </c>
       <c r="L52" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/amazon-fire-tv-stick-4K-select/dp/B0C6W3D4RM/ref=zg_bs_g_electronics_d_sccl_6/134-3113057-6761362</t>
+          <t>https://www.amazon.com/amazon-fire-tv-stick-4K-select/dp/B0C6W3D4RM/ref=zg_bs_g_electronics_d_sccl_6/134-1095087-0412057</t>
         </is>
       </c>
     </row>
@@ -9590,7 +9590,7 @@
       </c>
       <c r="B60" s="4" t="inlineStr">
         <is>
-          <t>xrp price</t>
+          <t>dave franco</t>
         </is>
       </c>
       <c r="C60" s="4" t="inlineStr">
@@ -9600,17 +9600,17 @@
       </c>
       <c r="D60" s="4" t="inlineStr">
         <is>
-          <t>Beauty &amp; Personal Care</t>
+          <t>Pet Supplies</t>
         </is>
       </c>
       <c r="E60" s="3" t="n">
-        <v>63.2</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="F60" s="3" t="n">
         <v>78</v>
       </c>
       <c r="G60" s="3" t="n">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="H60" s="3" t="inlineStr">
         <is>
@@ -9629,12 +9629,12 @@
       </c>
       <c r="K60" s="4" t="inlineStr">
         <is>
-          <t>TikTok Made Me Buy It / Honest Review</t>
+          <t>Emotional Reaction &amp; Satisfying Fur Release ASMR</t>
         </is>
       </c>
       <c r="L60" s="5" t="inlineStr">
         <is>
-          <t>https://trends.google.com/trends/explore?geo=US&amp;q=xrp%20price</t>
+          <t>https://trends.google.com/trends/explore?geo=US&amp;q=dave%20franco</t>
         </is>
       </c>
     </row>
@@ -9644,7 +9644,7 @@
       </c>
       <c r="B61" s="4" t="inlineStr">
         <is>
-          <t>omaha weather</t>
+          <t>goog stock</t>
         </is>
       </c>
       <c r="C61" s="4" t="inlineStr">
@@ -9688,7 +9688,7 @@
       </c>
       <c r="L61" s="5" t="inlineStr">
         <is>
-          <t>https://trends.google.com/trends/explore?geo=US&amp;q=omaha%20weather</t>
+          <t>https://trends.google.com/trends/explore?geo=US&amp;q=goog%20stock</t>
         </is>
       </c>
     </row>
@@ -9698,7 +9698,7 @@
       </c>
       <c r="B62" s="4" t="inlineStr">
         <is>
-          <t>oil prices</t>
+          <t>aaron gordon</t>
         </is>
       </c>
       <c r="C62" s="4" t="inlineStr">
@@ -9737,12 +9737,12 @@
       </c>
       <c r="K62" s="4" t="inlineStr">
         <is>
-          <t>Before/After Macro Skin Texture Zoom (Cận cảnh bề mặt da)</t>
+          <t>TikTok Made Me Buy It / Honest Review</t>
         </is>
       </c>
       <c r="L62" s="5" t="inlineStr">
         <is>
-          <t>https://trends.google.com/trends/explore?geo=US&amp;q=oil%20prices</t>
+          <t>https://trends.google.com/trends/explore?geo=US&amp;q=aaron%20gordon</t>
         </is>
       </c>
     </row>
@@ -9752,7 +9752,7 @@
       </c>
       <c r="B63" s="4" t="inlineStr">
         <is>
-          <t>temperature</t>
+          <t>todd blanche joe digenova call</t>
         </is>
       </c>
       <c r="C63" s="4" t="inlineStr">
@@ -9762,7 +9762,7 @@
       </c>
       <c r="D63" s="4" t="inlineStr">
         <is>
-          <t>DIY, Craft &amp; POD</t>
+          <t>Gadgets &amp; Electronics</t>
         </is>
       </c>
       <c r="E63" s="3" t="n">
@@ -9791,12 +9791,12 @@
       </c>
       <c r="K63" s="4" t="inlineStr">
         <is>
-          <t>Behind The Scenes Crafting &amp; Emotional Gift Unboxing</t>
+          <t>TikTok Made Me Buy It / Honest Review</t>
         </is>
       </c>
       <c r="L63" s="5" t="inlineStr">
         <is>
-          <t>https://trends.google.com/trends/explore?geo=US&amp;q=temperature</t>
+          <t>https://trends.google.com/trends/explore?geo=US&amp;q=todd%20blanche%20joe%20digenova%20call</t>
         </is>
       </c>
     </row>
@@ -9806,7 +9806,7 @@
       </c>
       <c r="B64" s="4" t="inlineStr">
         <is>
-          <t>clarity act</t>
+          <t>tropical storm weather forecast</t>
         </is>
       </c>
       <c r="C64" s="4" t="inlineStr">
@@ -9816,7 +9816,7 @@
       </c>
       <c r="D64" s="4" t="inlineStr">
         <is>
-          <t>DIY, Craft &amp; POD</t>
+          <t>Beauty &amp; Personal Care</t>
         </is>
       </c>
       <c r="E64" s="3" t="n">
@@ -9845,12 +9845,12 @@
       </c>
       <c r="K64" s="4" t="inlineStr">
         <is>
-          <t>Behind The Scenes Crafting &amp; Emotional Gift Unboxing</t>
+          <t>TikTok Made Me Buy It / Honest Review</t>
         </is>
       </c>
       <c r="L64" s="5" t="inlineStr">
         <is>
-          <t>https://trends.google.com/trends/explore?geo=US&amp;q=clarity%20act</t>
+          <t>https://trends.google.com/trends/explore?geo=US&amp;q=tropical%20storm%20weather%20forecast</t>
         </is>
       </c>
     </row>
@@ -9860,7 +9860,7 @@
       </c>
       <c r="B65" s="4" t="inlineStr">
         <is>
-          <t>npr</t>
+          <t>nvda</t>
         </is>
       </c>
       <c r="C65" s="4" t="inlineStr">
@@ -9904,7 +9904,7 @@
       </c>
       <c r="L65" s="5" t="inlineStr">
         <is>
-          <t>https://trends.google.com/trends/explore?geo=US&amp;q=npr</t>
+          <t>https://trends.google.com/trends/explore?geo=US&amp;q=nvda</t>
         </is>
       </c>
     </row>
@@ -9914,7 +9914,7 @@
       </c>
       <c r="B66" s="4" t="inlineStr">
         <is>
-          <t>kaley cuoco</t>
+          <t>omaha weather</t>
         </is>
       </c>
       <c r="C66" s="4" t="inlineStr">
@@ -9958,7 +9958,7 @@
       </c>
       <c r="L66" s="5" t="inlineStr">
         <is>
-          <t>https://trends.google.com/trends/explore?geo=US&amp;q=kaley%20cuoco</t>
+          <t>https://trends.google.com/trends/explore?geo=US&amp;q=omaha%20weather</t>
         </is>
       </c>
     </row>
@@ -9968,7 +9968,7 @@
       </c>
       <c r="B67" s="4" t="inlineStr">
         <is>
-          <t>reba mcentire dolly parton emmy tribute</t>
+          <t>xrp price</t>
         </is>
       </c>
       <c r="C67" s="4" t="inlineStr">
@@ -9978,7 +9978,7 @@
       </c>
       <c r="D67" s="4" t="inlineStr">
         <is>
-          <t>DIY, Craft &amp; POD</t>
+          <t>Beauty &amp; Personal Care</t>
         </is>
       </c>
       <c r="E67" s="3" t="n">
@@ -10007,12 +10007,12 @@
       </c>
       <c r="K67" s="4" t="inlineStr">
         <is>
-          <t>Behind The Scenes Crafting &amp; Emotional Gift Unboxing</t>
+          <t>TikTok Made Me Buy It / Honest Review</t>
         </is>
       </c>
       <c r="L67" s="5" t="inlineStr">
         <is>
-          <t>https://trends.google.com/trends/explore?geo=US&amp;q=reba%20mcentire%20dolly%20parton%20emmy%20tribute</t>
+          <t>https://trends.google.com/trends/explore?geo=US&amp;q=xrp%20price</t>
         </is>
       </c>
     </row>
@@ -10022,7 +10022,7 @@
       </c>
       <c r="B68" s="4" t="inlineStr">
         <is>
-          <t>erin napier</t>
+          <t>clarity act</t>
         </is>
       </c>
       <c r="C68" s="4" t="inlineStr">
@@ -10066,7 +10066,7 @@
       </c>
       <c r="L68" s="5" t="inlineStr">
         <is>
-          <t>https://trends.google.com/trends/explore?geo=US&amp;q=erin%20napier</t>
+          <t>https://trends.google.com/trends/explore?geo=US&amp;q=clarity%20act</t>
         </is>
       </c>
     </row>
@@ -10076,7 +10076,7 @@
       </c>
       <c r="B69" s="4" t="inlineStr">
         <is>
-          <t>blake lively</t>
+          <t>temperature</t>
         </is>
       </c>
       <c r="C69" s="4" t="inlineStr">
@@ -10086,7 +10086,7 @@
       </c>
       <c r="D69" s="4" t="inlineStr">
         <is>
-          <t>Beauty &amp; Personal Care</t>
+          <t>DIY, Craft &amp; POD</t>
         </is>
       </c>
       <c r="E69" s="3" t="n">
@@ -10115,12 +10115,12 @@
       </c>
       <c r="K69" s="4" t="inlineStr">
         <is>
-          <t>TikTok Made Me Buy It / Honest Review</t>
+          <t>Behind The Scenes Crafting &amp; Emotional Gift Unboxing</t>
         </is>
       </c>
       <c r="L69" s="5" t="inlineStr">
         <is>
-          <t>https://trends.google.com/trends/explore?geo=US&amp;q=blake%20lively</t>
+          <t>https://trends.google.com/trends/explore?geo=US&amp;q=temperature</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: resolve broken video links, fix KOL handles and avatars, add searchByKeyword handler, and display full 100 ranks with Supabase sync
</commit_message>
<xml_diff>
--- a/exports/TikTok_Shop_US_Latest_Trends.xlsx
+++ b/exports/TikTok_Shop_US_Latest_Trends.xlsx
@@ -1410,7 +1410,7 @@
       </c>
       <c r="J21" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/STANLEY-Quencher-State-Tumbler-Quartz/dp/B0CP9Z56SW/ref=zg_bs_g_kitchen_d_sccl_2/134-1095087-0412057</t>
+          <t>https://www.amazon.com/STANLEY-Quencher-State-Tumbler-Quartz/dp/B0CP9Z56SW/ref=zg_bs_g_kitchen_d_sccl_2/143-7478900-6733836</t>
         </is>
       </c>
     </row>
@@ -1456,7 +1456,7 @@
       </c>
       <c r="J22" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/Medicube-Zero-Pore-Pads-Dual-Textured/dp/B09V7Z4TJG/ref=zg_bs_g_beauty_d_sccl_2/134-1095087-0412057</t>
+          <t>https://www.amazon.com/Medicube-Zero-Pore-Pads-Dual-Textured/dp/B09V7Z4TJG/ref=zg_bs_g_beauty_d_sccl_2/143-7478900-6733836</t>
         </is>
       </c>
     </row>
@@ -1502,7 +1502,7 @@
       </c>
       <c r="J23" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/HydroJug-Traveler-Resistant-Bottle-Reusable-Insulated/dp/B0CQVWT2NH/ref=zg_bs_g_kitchen_d_sccl_3/134-1095087-0412057</t>
+          <t>https://www.amazon.com/HydroJug-Traveler-Resistant-Bottle-Reusable-Insulated/dp/B0CQVWT2NH/ref=zg_bs_g_kitchen_d_sccl_3/143-7478900-6733836</t>
         </is>
       </c>
     </row>
@@ -1590,7 +1590,7 @@
       </c>
       <c r="J25" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/Apple-EarPods-Headphones-Built-Control/dp/B0DCH8VDXF/ref=zg_bs_g_electronics_d_sccl_2/134-1095087-0412057</t>
+          <t>https://www.amazon.com/Apple-EarPods-Headphones-Built-Control/dp/B0DCH8VDXF/ref=zg_bs_g_electronics_d_sccl_2/143-7478900-6733836</t>
         </is>
       </c>
     </row>
@@ -1636,7 +1636,7 @@
       </c>
       <c r="J26" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/Apple-AirTag-2nd-Generation-Precision/dp/B0GJTFXNRX/ref=zg_bs_g_electronics_d_sccl_3/134-1095087-0412057</t>
+          <t>https://www.amazon.com/Apple-AirTag-2nd-Generation-Precision/dp/B0GJTFXNRX/ref=zg_bs_g_electronics_d_sccl_3/143-7478900-6733836</t>
         </is>
       </c>
     </row>
@@ -1724,7 +1724,7 @@
       </c>
       <c r="J28" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/Apple-Cancellation-Translation-Headphones-High-Fidelity/dp/B0FQFB8FMG/ref=zg_bs_g_electronics_d_sccl_4/134-1095087-0412057</t>
+          <t>https://www.amazon.com/Apple-Cancellation-Translation-Headphones-High-Fidelity/dp/B0FQFB8FMG/ref=zg_bs_g_electronics_d_sccl_4/143-7478900-6733836</t>
         </is>
       </c>
     </row>
@@ -1770,7 +1770,7 @@
       </c>
       <c r="J29" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/Roku-Streaming-Stick-HD-2025/dp/B0DXXYS4BJ/ref=zg_bs_g_electronics_d_sccl_5/134-1095087-0412057</t>
+          <t>https://www.amazon.com/Roku-Streaming-Stick-HD-2025/dp/B0DXXYS4BJ/ref=zg_bs_g_electronics_d_sccl_5/143-7478900-6733836</t>
         </is>
       </c>
     </row>
@@ -1816,7 +1816,7 @@
       </c>
       <c r="J30" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/amazon-fire-tv-stick-4K-select/dp/B0C6W3D4RM/ref=zg_bs_g_electronics_d_sccl_6/134-1095087-0412057</t>
+          <t>https://www.amazon.com/amazon-fire-tv-stick-4K-select/dp/B0C6W3D4RM/ref=zg_bs_g_electronics_d_sccl_6/143-7478900-6733836</t>
         </is>
       </c>
     </row>
@@ -2174,7 +2174,7 @@
       </c>
       <c r="B39" s="4" t="inlineStr">
         <is>
-          <t>goog stock</t>
+          <t>hugging face incident</t>
         </is>
       </c>
       <c r="C39" s="4" t="inlineStr">
@@ -2210,7 +2210,7 @@
       </c>
       <c r="J39" s="5" t="inlineStr">
         <is>
-          <t>https://trends.google.com/trends/explore?geo=US&amp;q=goog%20stock</t>
+          <t>https://trends.google.com/trends/explore?geo=US&amp;q=hugging%20face%20incident</t>
         </is>
       </c>
     </row>
@@ -2220,12 +2220,12 @@
       </c>
       <c r="B40" s="4" t="inlineStr">
         <is>
-          <t>aaron gordon</t>
+          <t>michael j fox</t>
         </is>
       </c>
       <c r="C40" s="4" t="inlineStr">
         <is>
-          <t>Beauty &amp; Personal Care</t>
+          <t>Phones &amp; Electronics</t>
         </is>
       </c>
       <c r="D40" s="3" t="n">
@@ -2246,17 +2246,17 @@
       </c>
       <c r="H40" s="4" t="inlineStr">
         <is>
-          <t>Đặt câu hỏi trúng nỗi đau thường ngày: 'Tại sao không ai nói cho tôi biết món đồ này sớm hơn?!'</t>
+          <t>So sánh âm thanh: 'Bật lọc tạp âm và nói chuyện giữa chợ ồn ào xem micro này xịn cỡ nào!'</t>
         </is>
       </c>
       <c r="I40" s="4" t="inlineStr">
         <is>
-          <t>Khách hàng mua sắm ngẫu hứng (Impulse Buyers) trên TikTok Shop US độ tuổi 18 - 45.</t>
+          <t>Học sinh, Gen Z làm bullet journal, Content Creator quay video TikTok / Vlog tại US.</t>
         </is>
       </c>
       <c r="J40" s="5" t="inlineStr">
         <is>
-          <t>https://trends.google.com/trends/explore?geo=US&amp;q=aaron%20gordon</t>
+          <t>https://trends.google.com/trends/explore?geo=US&amp;q=michael%20j%20fox</t>
         </is>
       </c>
     </row>
@@ -2266,12 +2266,12 @@
       </c>
       <c r="B41" s="4" t="inlineStr">
         <is>
-          <t>todd blanche joe digenova call</t>
+          <t>oracle layoffs</t>
         </is>
       </c>
       <c r="C41" s="4" t="inlineStr">
         <is>
-          <t>Gadgets &amp; Electronics</t>
+          <t>Beauty &amp; Personal Care</t>
         </is>
       </c>
       <c r="D41" s="3" t="n">
@@ -2302,7 +2302,7 @@
       </c>
       <c r="J41" s="5" t="inlineStr">
         <is>
-          <t>https://trends.google.com/trends/explore?geo=US&amp;q=todd%20blanche%20joe%20digenova%20call</t>
+          <t>https://trends.google.com/trends/explore?geo=US&amp;q=oracle%20layoffs</t>
         </is>
       </c>
     </row>
@@ -2312,7 +2312,7 @@
       </c>
       <c r="B42" s="4" t="inlineStr">
         <is>
-          <t>tropical storm weather forecast</t>
+          <t>mta</t>
         </is>
       </c>
       <c r="C42" s="4" t="inlineStr">
@@ -2338,17 +2338,17 @@
       </c>
       <c r="H42" s="4" t="inlineStr">
         <is>
-          <t>Đặt câu hỏi trúng nỗi đau thường ngày: 'Tại sao không ai nói cho tôi biết món đồ này sớm hơn?!'</t>
+          <t>Before &amp; After cận cảnh lỗ chân lông: 'Dừng ngay nếu bạn vẫn đang nặn mụn hoặc dùng tẩy tế bào chết hạt to!'</t>
         </is>
       </c>
       <c r="I42" s="4" t="inlineStr">
         <is>
-          <t>Khách hàng mua sắm ngẫu hứng (Impulse Buyers) trên TikTok Shop US độ tuổi 18 - 45.</t>
+          <t>Gen Z &amp; Millennials (18-34 tuổi), Chăm sóc da mụn, tín đồ Skincare &amp; 'Clean Girl' aesthetic US.</t>
         </is>
       </c>
       <c r="J42" s="5" t="inlineStr">
         <is>
-          <t>https://trends.google.com/trends/explore?geo=US&amp;q=tropical%20storm%20weather%20forecast</t>
+          <t>https://trends.google.com/trends/explore?geo=US&amp;q=mta</t>
         </is>
       </c>
     </row>
@@ -2358,7 +2358,7 @@
       </c>
       <c r="B43" s="4" t="inlineStr">
         <is>
-          <t>nvda</t>
+          <t>goog stock</t>
         </is>
       </c>
       <c r="C43" s="4" t="inlineStr">
@@ -2394,7 +2394,7 @@
       </c>
       <c r="J43" s="5" t="inlineStr">
         <is>
-          <t>https://trends.google.com/trends/explore?geo=US&amp;q=nvda</t>
+          <t>https://trends.google.com/trends/explore?geo=US&amp;q=goog%20stock</t>
         </is>
       </c>
     </row>
@@ -2404,7 +2404,7 @@
       </c>
       <c r="B44" s="4" t="inlineStr">
         <is>
-          <t>omaha weather</t>
+          <t>aaron gordon</t>
         </is>
       </c>
       <c r="C44" s="4" t="inlineStr">
@@ -2440,7 +2440,7 @@
       </c>
       <c r="J44" s="5" t="inlineStr">
         <is>
-          <t>https://trends.google.com/trends/explore?geo=US&amp;q=omaha%20weather</t>
+          <t>https://trends.google.com/trends/explore?geo=US&amp;q=aaron%20gordon</t>
         </is>
       </c>
     </row>
@@ -2450,12 +2450,12 @@
       </c>
       <c r="B45" s="4" t="inlineStr">
         <is>
-          <t>xrp price</t>
+          <t>todd blanche joe digenova call</t>
         </is>
       </c>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t>Beauty &amp; Personal Care</t>
+          <t>Gadgets &amp; Electronics</t>
         </is>
       </c>
       <c r="D45" s="3" t="n">
@@ -2486,7 +2486,7 @@
       </c>
       <c r="J45" s="5" t="inlineStr">
         <is>
-          <t>https://trends.google.com/trends/explore?geo=US&amp;q=xrp%20price</t>
+          <t>https://trends.google.com/trends/explore?geo=US&amp;q=todd%20blanche%20joe%20digenova%20call</t>
         </is>
       </c>
     </row>
@@ -2496,7 +2496,7 @@
       </c>
       <c r="B46" s="4" t="inlineStr">
         <is>
-          <t>clarity act</t>
+          <t>tropical storm weather forecast</t>
         </is>
       </c>
       <c r="C46" s="4" t="inlineStr">
@@ -2532,7 +2532,7 @@
       </c>
       <c r="J46" s="5" t="inlineStr">
         <is>
-          <t>https://trends.google.com/trends/explore?geo=US&amp;q=clarity%20act</t>
+          <t>https://trends.google.com/trends/explore?geo=US&amp;q=tropical%20storm%20weather%20forecast</t>
         </is>
       </c>
     </row>
@@ -2542,12 +2542,12 @@
       </c>
       <c r="B47" s="4" t="inlineStr">
         <is>
-          <t>temperature</t>
+          <t>dominick bianchi</t>
         </is>
       </c>
       <c r="C47" s="4" t="inlineStr">
         <is>
-          <t>DIY, Craft &amp; POD</t>
+          <t>Beauty &amp; Personal Care</t>
         </is>
       </c>
       <c r="D47" s="3" t="n">
@@ -2568,17 +2568,17 @@
       </c>
       <c r="H47" s="4" t="inlineStr">
         <is>
-          <t>Quá trình máy khắc laser tên khách hàng lên gỗ/kim loại: 'Làm món quà độc nhất vô nhị tặng mẹ...'</t>
+          <t>Đặt câu hỏi trúng nỗi đau thường ngày: 'Tại sao không ai nói cho tôi biết món đồ này sớm hơn?!'</t>
         </is>
       </c>
       <c r="I47" s="4" t="inlineStr">
         <is>
-          <t>Người tìm quà tặng sinh nhật, kỷ niệm, Mother's Day, quà tân gia ý nghĩa quanh năm.</t>
+          <t>Khách hàng mua sắm ngẫu hứng (Impulse Buyers) trên TikTok Shop US độ tuổi 18 - 45.</t>
         </is>
       </c>
       <c r="J47" s="5" t="inlineStr">
         <is>
-          <t>https://trends.google.com/trends/explore?geo=US&amp;q=temperature</t>
+          <t>https://trends.google.com/trends/explore?geo=US&amp;q=dominick%20bianchi</t>
         </is>
       </c>
     </row>
@@ -5257,7 +5257,7 @@
       </c>
       <c r="I3" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/eos-Cashmere-Moisture-Lightweight-Non-Greasy/dp/B08KT2Z93D/ref=zg_bs_g_beauty_d_sccl_1/134-1095087-0412057</t>
+          <t>https://www.amazon.com/eos-Cashmere-Moisture-Lightweight-Non-Greasy/dp/B08KT2Z93D/ref=zg_bs_g_beauty_d_sccl_1/143-7478900-6733836</t>
         </is>
       </c>
     </row>
@@ -5298,7 +5298,7 @@
       </c>
       <c r="I4" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/Mighty-Patch-Hydrocolloid-Absorbing-count/dp/B074PVTPBW/ref=zg_bs_g_beauty_d_sccl_5/134-1095087-0412057</t>
+          <t>https://www.amazon.com/Mighty-Patch-Hydrocolloid-Absorbing-count/dp/B074PVTPBW/ref=zg_bs_g_beauty_d_sccl_5/143-7478900-6733836</t>
         </is>
       </c>
     </row>
@@ -5339,7 +5339,7 @@
       </c>
       <c r="I5" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/TERRO-T300-2-2-Pack-Liquid-Baits/dp/B00E4GACB8/ref=zg_bs_g_home-garden_d_sccl_1/134-1095087-0412057</t>
+          <t>https://www.amazon.com/TERRO-T300-2-2-Pack-Liquid-Baits/dp/B00E4GACB8/ref=zg_bs_g_home-garden_d_sccl_1/143-7478900-6733836</t>
         </is>
       </c>
     </row>
@@ -5380,7 +5380,7 @@
       </c>
       <c r="I6" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/Queen-Size-Piece-Sheet-Set/dp/B01M16WBW1/ref=zg_bs_g_home-garden_d_sccl_3/134-1095087-0412057</t>
+          <t>https://www.amazon.com/Queen-Size-Piece-Sheet-Set/dp/B01M16WBW1/ref=zg_bs_g_home-garden_d_sccl_3/143-7478900-6733836</t>
         </is>
       </c>
     </row>
@@ -5421,7 +5421,7 @@
       </c>
       <c r="I7" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/Dr-Elseys-Premium-Clumping-Litter/dp/B0009X29WK/ref=zg_bs_g_pet-supplies_d_sccl_1/134-1095087-0412057</t>
+          <t>https://www.amazon.com/Dr-Elseys-Premium-Clumping-Litter/dp/B0009X29WK/ref=zg_bs_g_pet-supplies_d_sccl_1/143-7478900-6733836</t>
         </is>
       </c>
     </row>
@@ -5462,7 +5462,7 @@
       </c>
       <c r="I8" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/Amazon-Basics-Leak-Proof-Quick-Dry-Absorbency/dp/B00MW8G62E/ref=zg_bs_g_pet-supplies_d_sccl_2/134-1095087-0412057</t>
+          <t>https://www.amazon.com/Amazon-Basics-Leak-Proof-Quick-Dry-Absorbency/dp/B00MW8G62E/ref=zg_bs_g_pet-supplies_d_sccl_2/143-7478900-6733836</t>
         </is>
       </c>
     </row>
@@ -5503,7 +5503,7 @@
       </c>
       <c r="I9" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/Purina-Fancy-Feast-Poultry-Collection/dp/B00JN9IWNG/ref=zg_bs_g_pet-supplies_d_sccl_3/134-1095087-0412057</t>
+          <t>https://www.amazon.com/Purina-Fancy-Feast-Poultry-Collection/dp/B00JN9IWNG/ref=zg_bs_g_pet-supplies_d_sccl_3/143-7478900-6733836</t>
         </is>
       </c>
     </row>
@@ -5544,7 +5544,7 @@
       </c>
       <c r="I10" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/Amazon-Basics-Cotton-Swabs-500ct/dp/B09541P9WH/ref=zg_bs_g_beauty_d_sccl_3/134-1095087-0412057</t>
+          <t>https://www.amazon.com/Amazon-Basics-Cotton-Swabs-500ct/dp/B09541P9WH/ref=zg_bs_g_beauty_d_sccl_3/143-7478900-6733836</t>
         </is>
       </c>
     </row>
@@ -5585,7 +5585,7 @@
       </c>
       <c r="I11" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/Clean-Skin-Club-Disposable-Sensitive/dp/B07PBXXNCY/ref=zg_bs_g_beauty_d_sccl_4/134-1095087-0412057</t>
+          <t>https://www.amazon.com/Clean-Skin-Club-Disposable-Sensitive/dp/B07PBXXNCY/ref=zg_bs_g_beauty_d_sccl_4/143-7478900-6733836</t>
         </is>
       </c>
     </row>
@@ -5626,7 +5626,7 @@
       </c>
       <c r="I12" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/Owala-FreeSip-Insulated-Stainless-BPA-Free/dp/B0BZYCJK89/ref=zg_bs_g_kitchen_d_sccl_1/134-1095087-0412057</t>
+          <t>https://www.amazon.com/Owala-FreeSip-Insulated-Stainless-BPA-Free/dp/B0BZYCJK89/ref=zg_bs_g_kitchen_d_sccl_1/143-7478900-6733836</t>
         </is>
       </c>
     </row>
@@ -5667,7 +5667,7 @@
       </c>
       <c r="I13" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/Owala-FreeSip-Insulated-Stainless-BPA-Free/dp/B0BZYCJK89/ref=zg_bs_g_home-garden_d_sccl_2/134-1095087-0412057</t>
+          <t>https://www.amazon.com/Owala-FreeSip-Insulated-Stainless-BPA-Free/dp/B0BZYCJK89/ref=zg_bs_g_home-garden_d_sccl_2/143-7478900-6733836</t>
         </is>
       </c>
     </row>
@@ -5708,7 +5708,7 @@
       </c>
       <c r="I14" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/Blink-Plus-Plan-monthly-auto-renewal/dp/B08JHCVHTY/ref=zg_bs_g_electronics_d_sccl_1/134-1095087-0412057</t>
+          <t>https://www.amazon.com/Blink-Plus-Plan-monthly-auto-renewal/dp/B08JHCVHTY/ref=zg_bs_g_electronics_d_sccl_1/143-7478900-6733836</t>
         </is>
       </c>
     </row>
@@ -5749,7 +5749,7 @@
       </c>
       <c r="I15" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/Owala-SmoothSip-Insulated-Stainless-Reusable/dp/B0DF3M7V3T/ref=zg_bs_g_kitchen_d_sccl_5/134-1095087-0412057</t>
+          <t>https://www.amazon.com/Owala-SmoothSip-Insulated-Stainless-Reusable/dp/B0DF3M7V3T/ref=zg_bs_g_kitchen_d_sccl_5/143-7478900-6733836</t>
         </is>
       </c>
     </row>
@@ -5790,7 +5790,7 @@
       </c>
       <c r="I16" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/Amazon-Basics-Cotton-Rounds-Count/dp/B09542G9ZN/ref=zg_bs_g_beauty_d_sccl_6/134-1095087-0412057</t>
+          <t>https://www.amazon.com/Amazon-Basics-Cotton-Rounds-Count/dp/B09542G9ZN/ref=zg_bs_g_beauty_d_sccl_6/143-7478900-6733836</t>
         </is>
       </c>
     </row>
@@ -5831,7 +5831,7 @@
       </c>
       <c r="I17" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/Etekcity-Multifunction-Stainless-Batteries-Included/dp/B0113UZJE2/ref=zg_bs_g_kitchen_d_sccl_4/134-1095087-0412057</t>
+          <t>https://www.amazon.com/Etekcity-Multifunction-Stainless-Batteries-Included/dp/B0113UZJE2/ref=zg_bs_g_kitchen_d_sccl_4/143-7478900-6733836</t>
         </is>
       </c>
     </row>
@@ -5872,7 +5872,7 @@
       </c>
       <c r="I18" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/Amazon-Basics-Microfiber-Lightweight-Wrinkle-free/dp/B0154ASID6/ref=zg_bs_g_home-garden_d_sccl_4/134-1095087-0412057</t>
+          <t>https://www.amazon.com/Amazon-Basics-Microfiber-Lightweight-Wrinkle-free/dp/B0154ASID6/ref=zg_bs_g_home-garden_d_sccl_4/143-7478900-6733836</t>
         </is>
       </c>
     </row>
@@ -5913,7 +5913,7 @@
       </c>
       <c r="I19" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/Electric-Flying-Insect-Trap-Starter/dp/B07T869RNY/ref=zg_bs_g_home-garden_d_sccl_6/134-1095087-0412057</t>
+          <t>https://www.amazon.com/Electric-Flying-Insect-Trap-Starter/dp/B07T869RNY/ref=zg_bs_g_home-garden_d_sccl_6/143-7478900-6733836</t>
         </is>
       </c>
     </row>
@@ -5954,7 +5954,7 @@
       </c>
       <c r="I20" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/Earth-Rated-Lavender-Scented-Completely/dp/B00BSYR7K8/ref=zg_bs_g_pet-supplies_d_sccl_5/134-1095087-0412057</t>
+          <t>https://www.amazon.com/Earth-Rated-Lavender-Scented-Completely/dp/B00BSYR7K8/ref=zg_bs_g_pet-supplies_d_sccl_5/143-7478900-6733836</t>
         </is>
       </c>
     </row>
@@ -5995,7 +5995,7 @@
       </c>
       <c r="I21" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/Toaster-Fits-anywhereTM-Kitchenware-Setting-Removable/dp/B0CYJBB2JQ/ref=zg_bs_g_kitchen_d_sccl_6/134-1095087-0412057</t>
+          <t>https://www.amazon.com/Toaster-Fits-anywhereTM-Kitchenware-Setting-Removable/dp/B0CYJBB2JQ/ref=zg_bs_g_kitchen_d_sccl_6/143-7478900-6733836</t>
         </is>
       </c>
     </row>
@@ -6036,7 +6036,7 @@
       </c>
       <c r="I22" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/ZEVO-Flying-Insect-Refills-Indoor/dp/B0C3FTCYZL/ref=zg_bs_g_home-garden_d_sccl_5/134-1095087-0412057</t>
+          <t>https://www.amazon.com/ZEVO-Flying-Insect-Refills-Indoor/dp/B0C3FTCYZL/ref=zg_bs_g_home-garden_d_sccl_5/143-7478900-6733836</t>
         </is>
       </c>
     </row>
@@ -6077,7 +6077,7 @@
       </c>
       <c r="I23" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/INABA-Grain-Free-Lickable-Squeezable-Vitamin/dp/B0B52D7BBD/ref=zg_bs_g_pet-supplies_d_sccl_4/134-1095087-0412057</t>
+          <t>https://www.amazon.com/INABA-Grain-Free-Lickable-Squeezable-Vitamin/dp/B0B52D7BBD/ref=zg_bs_g_pet-supplies_d_sccl_4/143-7478900-6733836</t>
         </is>
       </c>
     </row>
@@ -6118,7 +6118,7 @@
       </c>
       <c r="I24" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/Greenies-Pill-Pockets-Ingredients-Nutrients/dp/B008GRONV6/ref=zg_bs_g_pet-supplies_d_sccl_6/134-1095087-0412057</t>
+          <t>https://www.amazon.com/Greenies-Pill-Pockets-Ingredients-Nutrients/dp/B008GRONV6/ref=zg_bs_g_pet-supplies_d_sccl_6/143-7478900-6733836</t>
         </is>
       </c>
     </row>
@@ -7556,7 +7556,7 @@
       </c>
       <c r="L21" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/STANLEY-Quencher-State-Tumbler-Quartz/dp/B0CP9Z56SW/ref=zg_bs_g_kitchen_d_sccl_2/134-1095087-0412057</t>
+          <t>https://www.amazon.com/STANLEY-Quencher-State-Tumbler-Quartz/dp/B0CP9Z56SW/ref=zg_bs_g_kitchen_d_sccl_2/143-7478900-6733836</t>
         </is>
       </c>
     </row>
@@ -7610,7 +7610,7 @@
       </c>
       <c r="L22" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/Medicube-Zero-Pore-Pads-Dual-Textured/dp/B09V7Z4TJG/ref=zg_bs_g_beauty_d_sccl_2/134-1095087-0412057</t>
+          <t>https://www.amazon.com/Medicube-Zero-Pore-Pads-Dual-Textured/dp/B09V7Z4TJG/ref=zg_bs_g_beauty_d_sccl_2/143-7478900-6733836</t>
         </is>
       </c>
     </row>
@@ -7664,7 +7664,7 @@
       </c>
       <c r="L23" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/HydroJug-Traveler-Resistant-Bottle-Reusable-Insulated/dp/B0CQVWT2NH/ref=zg_bs_g_kitchen_d_sccl_3/134-1095087-0412057</t>
+          <t>https://www.amazon.com/HydroJug-Traveler-Resistant-Bottle-Reusable-Insulated/dp/B0CQVWT2NH/ref=zg_bs_g_kitchen_d_sccl_3/143-7478900-6733836</t>
         </is>
       </c>
     </row>
@@ -7768,7 +7768,7 @@
       </c>
       <c r="L25" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/eos-Cashmere-Moisture-Lightweight-Non-Greasy/dp/B08KT2Z93D/ref=zg_bs_g_beauty_d_sccl_1/134-1095087-0412057</t>
+          <t>https://www.amazon.com/eos-Cashmere-Moisture-Lightweight-Non-Greasy/dp/B08KT2Z93D/ref=zg_bs_g_beauty_d_sccl_1/143-7478900-6733836</t>
         </is>
       </c>
     </row>
@@ -7822,7 +7822,7 @@
       </c>
       <c r="L26" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/Mighty-Patch-Hydrocolloid-Absorbing-count/dp/B074PVTPBW/ref=zg_bs_g_beauty_d_sccl_5/134-1095087-0412057</t>
+          <t>https://www.amazon.com/Mighty-Patch-Hydrocolloid-Absorbing-count/dp/B074PVTPBW/ref=zg_bs_g_beauty_d_sccl_5/143-7478900-6733836</t>
         </is>
       </c>
     </row>
@@ -7876,7 +7876,7 @@
       </c>
       <c r="L27" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/TERRO-T300-2-2-Pack-Liquid-Baits/dp/B00E4GACB8/ref=zg_bs_g_home-garden_d_sccl_1/134-1095087-0412057</t>
+          <t>https://www.amazon.com/TERRO-T300-2-2-Pack-Liquid-Baits/dp/B00E4GACB8/ref=zg_bs_g_home-garden_d_sccl_1/143-7478900-6733836</t>
         </is>
       </c>
     </row>
@@ -7930,7 +7930,7 @@
       </c>
       <c r="L28" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/Queen-Size-Piece-Sheet-Set/dp/B01M16WBW1/ref=zg_bs_g_home-garden_d_sccl_3/134-1095087-0412057</t>
+          <t>https://www.amazon.com/Queen-Size-Piece-Sheet-Set/dp/B01M16WBW1/ref=zg_bs_g_home-garden_d_sccl_3/143-7478900-6733836</t>
         </is>
       </c>
     </row>
@@ -7984,7 +7984,7 @@
       </c>
       <c r="L29" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/Dr-Elseys-Premium-Clumping-Litter/dp/B0009X29WK/ref=zg_bs_g_pet-supplies_d_sccl_1/134-1095087-0412057</t>
+          <t>https://www.amazon.com/Dr-Elseys-Premium-Clumping-Litter/dp/B0009X29WK/ref=zg_bs_g_pet-supplies_d_sccl_1/143-7478900-6733836</t>
         </is>
       </c>
     </row>
@@ -8038,7 +8038,7 @@
       </c>
       <c r="L30" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/Amazon-Basics-Leak-Proof-Quick-Dry-Absorbency/dp/B00MW8G62E/ref=zg_bs_g_pet-supplies_d_sccl_2/134-1095087-0412057</t>
+          <t>https://www.amazon.com/Amazon-Basics-Leak-Proof-Quick-Dry-Absorbency/dp/B00MW8G62E/ref=zg_bs_g_pet-supplies_d_sccl_2/143-7478900-6733836</t>
         </is>
       </c>
     </row>
@@ -8092,7 +8092,7 @@
       </c>
       <c r="L31" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/Purina-Fancy-Feast-Poultry-Collection/dp/B00JN9IWNG/ref=zg_bs_g_pet-supplies_d_sccl_3/134-1095087-0412057</t>
+          <t>https://www.amazon.com/Purina-Fancy-Feast-Poultry-Collection/dp/B00JN9IWNG/ref=zg_bs_g_pet-supplies_d_sccl_3/143-7478900-6733836</t>
         </is>
       </c>
     </row>
@@ -8146,7 +8146,7 @@
       </c>
       <c r="L32" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/Amazon-Basics-Cotton-Swabs-500ct/dp/B09541P9WH/ref=zg_bs_g_beauty_d_sccl_3/134-1095087-0412057</t>
+          <t>https://www.amazon.com/Amazon-Basics-Cotton-Swabs-500ct/dp/B09541P9WH/ref=zg_bs_g_beauty_d_sccl_3/143-7478900-6733836</t>
         </is>
       </c>
     </row>
@@ -8200,7 +8200,7 @@
       </c>
       <c r="L33" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/Clean-Skin-Club-Disposable-Sensitive/dp/B07PBXXNCY/ref=zg_bs_g_beauty_d_sccl_4/134-1095087-0412057</t>
+          <t>https://www.amazon.com/Clean-Skin-Club-Disposable-Sensitive/dp/B07PBXXNCY/ref=zg_bs_g_beauty_d_sccl_4/143-7478900-6733836</t>
         </is>
       </c>
     </row>
@@ -8254,7 +8254,7 @@
       </c>
       <c r="L34" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/Owala-FreeSip-Insulated-Stainless-BPA-Free/dp/B0BZYCJK89/ref=zg_bs_g_kitchen_d_sccl_1/134-1095087-0412057</t>
+          <t>https://www.amazon.com/Owala-FreeSip-Insulated-Stainless-BPA-Free/dp/B0BZYCJK89/ref=zg_bs_g_kitchen_d_sccl_1/143-7478900-6733836</t>
         </is>
       </c>
     </row>
@@ -8308,7 +8308,7 @@
       </c>
       <c r="L35" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/Owala-FreeSip-Insulated-Stainless-BPA-Free/dp/B0BZYCJK89/ref=zg_bs_g_home-garden_d_sccl_2/134-1095087-0412057</t>
+          <t>https://www.amazon.com/Owala-FreeSip-Insulated-Stainless-BPA-Free/dp/B0BZYCJK89/ref=zg_bs_g_home-garden_d_sccl_2/143-7478900-6733836</t>
         </is>
       </c>
     </row>
@@ -8362,7 +8362,7 @@
       </c>
       <c r="L36" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/Blink-Plus-Plan-monthly-auto-renewal/dp/B08JHCVHTY/ref=zg_bs_g_electronics_d_sccl_1/134-1095087-0412057</t>
+          <t>https://www.amazon.com/Blink-Plus-Plan-monthly-auto-renewal/dp/B08JHCVHTY/ref=zg_bs_g_electronics_d_sccl_1/143-7478900-6733836</t>
         </is>
       </c>
     </row>
@@ -8416,7 +8416,7 @@
       </c>
       <c r="L37" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/Owala-SmoothSip-Insulated-Stainless-Reusable/dp/B0DF3M7V3T/ref=zg_bs_g_kitchen_d_sccl_5/134-1095087-0412057</t>
+          <t>https://www.amazon.com/Owala-SmoothSip-Insulated-Stainless-Reusable/dp/B0DF3M7V3T/ref=zg_bs_g_kitchen_d_sccl_5/143-7478900-6733836</t>
         </is>
       </c>
     </row>
@@ -8470,7 +8470,7 @@
       </c>
       <c r="L38" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/Apple-EarPods-Headphones-Built-Control/dp/B0DCH8VDXF/ref=zg_bs_g_electronics_d_sccl_2/134-1095087-0412057</t>
+          <t>https://www.amazon.com/Apple-EarPods-Headphones-Built-Control/dp/B0DCH8VDXF/ref=zg_bs_g_electronics_d_sccl_2/143-7478900-6733836</t>
         </is>
       </c>
     </row>
@@ -8524,7 +8524,7 @@
       </c>
       <c r="L39" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/Apple-AirTag-2nd-Generation-Precision/dp/B0GJTFXNRX/ref=zg_bs_g_electronics_d_sccl_3/134-1095087-0412057</t>
+          <t>https://www.amazon.com/Apple-AirTag-2nd-Generation-Precision/dp/B0GJTFXNRX/ref=zg_bs_g_electronics_d_sccl_3/143-7478900-6733836</t>
         </is>
       </c>
     </row>
@@ -8628,7 +8628,7 @@
       </c>
       <c r="L41" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/Amazon-Basics-Cotton-Rounds-Count/dp/B09542G9ZN/ref=zg_bs_g_beauty_d_sccl_6/134-1095087-0412057</t>
+          <t>https://www.amazon.com/Amazon-Basics-Cotton-Rounds-Count/dp/B09542G9ZN/ref=zg_bs_g_beauty_d_sccl_6/143-7478900-6733836</t>
         </is>
       </c>
     </row>
@@ -8682,7 +8682,7 @@
       </c>
       <c r="L42" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/Etekcity-Multifunction-Stainless-Batteries-Included/dp/B0113UZJE2/ref=zg_bs_g_kitchen_d_sccl_4/134-1095087-0412057</t>
+          <t>https://www.amazon.com/Etekcity-Multifunction-Stainless-Batteries-Included/dp/B0113UZJE2/ref=zg_bs_g_kitchen_d_sccl_4/143-7478900-6733836</t>
         </is>
       </c>
     </row>
@@ -8736,7 +8736,7 @@
       </c>
       <c r="L43" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/Amazon-Basics-Microfiber-Lightweight-Wrinkle-free/dp/B0154ASID6/ref=zg_bs_g_home-garden_d_sccl_4/134-1095087-0412057</t>
+          <t>https://www.amazon.com/Amazon-Basics-Microfiber-Lightweight-Wrinkle-free/dp/B0154ASID6/ref=zg_bs_g_home-garden_d_sccl_4/143-7478900-6733836</t>
         </is>
       </c>
     </row>
@@ -8790,7 +8790,7 @@
       </c>
       <c r="L44" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/Electric-Flying-Insect-Trap-Starter/dp/B07T869RNY/ref=zg_bs_g_home-garden_d_sccl_6/134-1095087-0412057</t>
+          <t>https://www.amazon.com/Electric-Flying-Insect-Trap-Starter/dp/B07T869RNY/ref=zg_bs_g_home-garden_d_sccl_6/143-7478900-6733836</t>
         </is>
       </c>
     </row>
@@ -8844,7 +8844,7 @@
       </c>
       <c r="L45" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/Earth-Rated-Lavender-Scented-Completely/dp/B00BSYR7K8/ref=zg_bs_g_pet-supplies_d_sccl_5/134-1095087-0412057</t>
+          <t>https://www.amazon.com/Earth-Rated-Lavender-Scented-Completely/dp/B00BSYR7K8/ref=zg_bs_g_pet-supplies_d_sccl_5/143-7478900-6733836</t>
         </is>
       </c>
     </row>
@@ -8898,7 +8898,7 @@
       </c>
       <c r="L46" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/Toaster-Fits-anywhereTM-Kitchenware-Setting-Removable/dp/B0CYJBB2JQ/ref=zg_bs_g_kitchen_d_sccl_6/134-1095087-0412057</t>
+          <t>https://www.amazon.com/Toaster-Fits-anywhereTM-Kitchenware-Setting-Removable/dp/B0CYJBB2JQ/ref=zg_bs_g_kitchen_d_sccl_6/143-7478900-6733836</t>
         </is>
       </c>
     </row>
@@ -8952,7 +8952,7 @@
       </c>
       <c r="L47" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/ZEVO-Flying-Insect-Refills-Indoor/dp/B0C3FTCYZL/ref=zg_bs_g_home-garden_d_sccl_5/134-1095087-0412057</t>
+          <t>https://www.amazon.com/ZEVO-Flying-Insect-Refills-Indoor/dp/B0C3FTCYZL/ref=zg_bs_g_home-garden_d_sccl_5/143-7478900-6733836</t>
         </is>
       </c>
     </row>
@@ -9006,7 +9006,7 @@
       </c>
       <c r="L48" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/INABA-Grain-Free-Lickable-Squeezable-Vitamin/dp/B0B52D7BBD/ref=zg_bs_g_pet-supplies_d_sccl_4/134-1095087-0412057</t>
+          <t>https://www.amazon.com/INABA-Grain-Free-Lickable-Squeezable-Vitamin/dp/B0B52D7BBD/ref=zg_bs_g_pet-supplies_d_sccl_4/143-7478900-6733836</t>
         </is>
       </c>
     </row>
@@ -9060,7 +9060,7 @@
       </c>
       <c r="L49" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/Greenies-Pill-Pockets-Ingredients-Nutrients/dp/B008GRONV6/ref=zg_bs_g_pet-supplies_d_sccl_6/134-1095087-0412057</t>
+          <t>https://www.amazon.com/Greenies-Pill-Pockets-Ingredients-Nutrients/dp/B008GRONV6/ref=zg_bs_g_pet-supplies_d_sccl_6/143-7478900-6733836</t>
         </is>
       </c>
     </row>
@@ -9114,7 +9114,7 @@
       </c>
       <c r="L50" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/Apple-Cancellation-Translation-Headphones-High-Fidelity/dp/B0FQFB8FMG/ref=zg_bs_g_electronics_d_sccl_4/134-1095087-0412057</t>
+          <t>https://www.amazon.com/Apple-Cancellation-Translation-Headphones-High-Fidelity/dp/B0FQFB8FMG/ref=zg_bs_g_electronics_d_sccl_4/143-7478900-6733836</t>
         </is>
       </c>
     </row>
@@ -9168,7 +9168,7 @@
       </c>
       <c r="L51" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/Roku-Streaming-Stick-HD-2025/dp/B0DXXYS4BJ/ref=zg_bs_g_electronics_d_sccl_5/134-1095087-0412057</t>
+          <t>https://www.amazon.com/Roku-Streaming-Stick-HD-2025/dp/B0DXXYS4BJ/ref=zg_bs_g_electronics_d_sccl_5/143-7478900-6733836</t>
         </is>
       </c>
     </row>
@@ -9222,7 +9222,7 @@
       </c>
       <c r="L52" s="5" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/amazon-fire-tv-stick-4K-select/dp/B0C6W3D4RM/ref=zg_bs_g_electronics_d_sccl_6/134-1095087-0412057</t>
+          <t>https://www.amazon.com/amazon-fire-tv-stick-4K-select/dp/B0C6W3D4RM/ref=zg_bs_g_electronics_d_sccl_6/143-7478900-6733836</t>
         </is>
       </c>
     </row>
@@ -9644,7 +9644,7 @@
       </c>
       <c r="B61" s="4" t="inlineStr">
         <is>
-          <t>goog stock</t>
+          <t>hugging face incident</t>
         </is>
       </c>
       <c r="C61" s="4" t="inlineStr">
@@ -9688,7 +9688,7 @@
       </c>
       <c r="L61" s="5" t="inlineStr">
         <is>
-          <t>https://trends.google.com/trends/explore?geo=US&amp;q=goog%20stock</t>
+          <t>https://trends.google.com/trends/explore?geo=US&amp;q=hugging%20face%20incident</t>
         </is>
       </c>
     </row>
@@ -9698,7 +9698,7 @@
       </c>
       <c r="B62" s="4" t="inlineStr">
         <is>
-          <t>aaron gordon</t>
+          <t>michael j fox</t>
         </is>
       </c>
       <c r="C62" s="4" t="inlineStr">
@@ -9708,7 +9708,7 @@
       </c>
       <c r="D62" s="4" t="inlineStr">
         <is>
-          <t>Beauty &amp; Personal Care</t>
+          <t>Phones &amp; Electronics</t>
         </is>
       </c>
       <c r="E62" s="3" t="n">
@@ -9737,12 +9737,12 @@
       </c>
       <c r="K62" s="4" t="inlineStr">
         <is>
-          <t>TikTok Made Me Buy It / Honest Review</t>
+          <t>Side-by-side Live Demo &amp; Unboxing ASMR</t>
         </is>
       </c>
       <c r="L62" s="5" t="inlineStr">
         <is>
-          <t>https://trends.google.com/trends/explore?geo=US&amp;q=aaron%20gordon</t>
+          <t>https://trends.google.com/trends/explore?geo=US&amp;q=michael%20j%20fox</t>
         </is>
       </c>
     </row>
@@ -9752,7 +9752,7 @@
       </c>
       <c r="B63" s="4" t="inlineStr">
         <is>
-          <t>todd blanche joe digenova call</t>
+          <t>oracle layoffs</t>
         </is>
       </c>
       <c r="C63" s="4" t="inlineStr">
@@ -9762,7 +9762,7 @@
       </c>
       <c r="D63" s="4" t="inlineStr">
         <is>
-          <t>Gadgets &amp; Electronics</t>
+          <t>Beauty &amp; Personal Care</t>
         </is>
       </c>
       <c r="E63" s="3" t="n">
@@ -9796,7 +9796,7 @@
       </c>
       <c r="L63" s="5" t="inlineStr">
         <is>
-          <t>https://trends.google.com/trends/explore?geo=US&amp;q=todd%20blanche%20joe%20digenova%20call</t>
+          <t>https://trends.google.com/trends/explore?geo=US&amp;q=oracle%20layoffs</t>
         </is>
       </c>
     </row>
@@ -9806,7 +9806,7 @@
       </c>
       <c r="B64" s="4" t="inlineStr">
         <is>
-          <t>tropical storm weather forecast</t>
+          <t>mta</t>
         </is>
       </c>
       <c r="C64" s="4" t="inlineStr">
@@ -9845,12 +9845,12 @@
       </c>
       <c r="K64" s="4" t="inlineStr">
         <is>
-          <t>TikTok Made Me Buy It / Honest Review</t>
+          <t>Before/After Macro Skin Texture Zoom (Cận cảnh bề mặt da)</t>
         </is>
       </c>
       <c r="L64" s="5" t="inlineStr">
         <is>
-          <t>https://trends.google.com/trends/explore?geo=US&amp;q=tropical%20storm%20weather%20forecast</t>
+          <t>https://trends.google.com/trends/explore?geo=US&amp;q=mta</t>
         </is>
       </c>
     </row>
@@ -9860,7 +9860,7 @@
       </c>
       <c r="B65" s="4" t="inlineStr">
         <is>
-          <t>nvda</t>
+          <t>goog stock</t>
         </is>
       </c>
       <c r="C65" s="4" t="inlineStr">
@@ -9904,7 +9904,7 @@
       </c>
       <c r="L65" s="5" t="inlineStr">
         <is>
-          <t>https://trends.google.com/trends/explore?geo=US&amp;q=nvda</t>
+          <t>https://trends.google.com/trends/explore?geo=US&amp;q=goog%20stock</t>
         </is>
       </c>
     </row>
@@ -9914,7 +9914,7 @@
       </c>
       <c r="B66" s="4" t="inlineStr">
         <is>
-          <t>omaha weather</t>
+          <t>aaron gordon</t>
         </is>
       </c>
       <c r="C66" s="4" t="inlineStr">
@@ -9958,7 +9958,7 @@
       </c>
       <c r="L66" s="5" t="inlineStr">
         <is>
-          <t>https://trends.google.com/trends/explore?geo=US&amp;q=omaha%20weather</t>
+          <t>https://trends.google.com/trends/explore?geo=US&amp;q=aaron%20gordon</t>
         </is>
       </c>
     </row>
@@ -9968,7 +9968,7 @@
       </c>
       <c r="B67" s="4" t="inlineStr">
         <is>
-          <t>xrp price</t>
+          <t>todd blanche joe digenova call</t>
         </is>
       </c>
       <c r="C67" s="4" t="inlineStr">
@@ -9978,7 +9978,7 @@
       </c>
       <c r="D67" s="4" t="inlineStr">
         <is>
-          <t>Beauty &amp; Personal Care</t>
+          <t>Gadgets &amp; Electronics</t>
         </is>
       </c>
       <c r="E67" s="3" t="n">
@@ -10012,7 +10012,7 @@
       </c>
       <c r="L67" s="5" t="inlineStr">
         <is>
-          <t>https://trends.google.com/trends/explore?geo=US&amp;q=xrp%20price</t>
+          <t>https://trends.google.com/trends/explore?geo=US&amp;q=todd%20blanche%20joe%20digenova%20call</t>
         </is>
       </c>
     </row>
@@ -10022,7 +10022,7 @@
       </c>
       <c r="B68" s="4" t="inlineStr">
         <is>
-          <t>clarity act</t>
+          <t>tropical storm weather forecast</t>
         </is>
       </c>
       <c r="C68" s="4" t="inlineStr">
@@ -10066,7 +10066,7 @@
       </c>
       <c r="L68" s="5" t="inlineStr">
         <is>
-          <t>https://trends.google.com/trends/explore?geo=US&amp;q=clarity%20act</t>
+          <t>https://trends.google.com/trends/explore?geo=US&amp;q=tropical%20storm%20weather%20forecast</t>
         </is>
       </c>
     </row>
@@ -10076,7 +10076,7 @@
       </c>
       <c r="B69" s="4" t="inlineStr">
         <is>
-          <t>temperature</t>
+          <t>dominick bianchi</t>
         </is>
       </c>
       <c r="C69" s="4" t="inlineStr">
@@ -10086,7 +10086,7 @@
       </c>
       <c r="D69" s="4" t="inlineStr">
         <is>
-          <t>DIY, Craft &amp; POD</t>
+          <t>Beauty &amp; Personal Care</t>
         </is>
       </c>
       <c r="E69" s="3" t="n">
@@ -10115,12 +10115,12 @@
       </c>
       <c r="K69" s="4" t="inlineStr">
         <is>
-          <t>Behind The Scenes Crafting &amp; Emotional Gift Unboxing</t>
+          <t>TikTok Made Me Buy It / Honest Review</t>
         </is>
       </c>
       <c r="L69" s="5" t="inlineStr">
         <is>
-          <t>https://trends.google.com/trends/explore?geo=US&amp;q=temperature</t>
+          <t>https://trends.google.com/trends/explore?geo=US&amp;q=dominick%20bianchi</t>
         </is>
       </c>
     </row>
@@ -13723,7 +13723,7 @@
       </c>
       <c r="L3" s="5" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@thebeachwaver/video/741982736192</t>
+          <t>https://www.tiktok.com/search?q=Beachwaver%20S1.25%20Dual%20Voltage%20Automatic%20Rotating%20Ceramic%20Curling%20Wand</t>
         </is>
       </c>
     </row>
@@ -13781,7 +13781,7 @@
       </c>
       <c r="L4" s="5" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@cleanwithme_asmr/video/7410982736192</t>
+          <t>https://www.tiktok.com/search?q=thebeachwaver%20Electric%20Spin%20Scrubber%20360%20Cordless%20Power%20Shower%20Cleaner%20Brush</t>
         </is>
       </c>
     </row>
@@ -13811,7 +13811,7 @@
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>@owala_official</t>
+          <t>@owalalife</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
@@ -13839,7 +13839,7 @@
       </c>
       <c r="L5" s="5" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@owala_official/video/749982736192</t>
+          <t>https://www.tiktok.com/search?q=cleanwithme_asmr%20Owala%20FreeSip%2032oz%20Insulated%20Stainless%20Steel%20Water%20Bottle%20Tumbler</t>
         </is>
       </c>
     </row>
@@ -13869,7 +13869,7 @@
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>@keychron_official</t>
+          <t>@keychron</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr">
@@ -13897,7 +13897,7 @@
       </c>
       <c r="L6" s="5" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@keychron_official/video/7415982736192</t>
+          <t>https://www.tiktok.com/search?q=owalalife%20Wireless%20Custom%20Mechanical%20Keyboard%20RGB%20Hot-Swappable%20Gateron%20Pro</t>
         </is>
       </c>
     </row>
@@ -13955,7 +13955,7 @@
       </c>
       <c r="L7" s="5" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@ergonomic_living/video/7418982736192</t>
+          <t>https://www.tiktok.com/search?q=keychron%20Breathable%20Mesh%20Ergonomic%20Office%20Chair%20with%203D%20Lumbar%20Support</t>
         </is>
       </c>
     </row>
@@ -14013,7 +14013,7 @@
       </c>
       <c r="L8" s="5" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@thebeachwaver/video/7534817293019</t>
+          <t>https://www.tiktok.com/search?q=ergonomic_living%20Beachwaver%20S1.25%20Dual%20Voltage%20Automatic%20Rotating%20Ceramic%20Curling%20Wand</t>
         </is>
       </c>
     </row>
@@ -14071,7 +14071,7 @@
       </c>
       <c r="L9" s="5" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@led_vibes_room/video/7420982736192</t>
+          <t>https://www.tiktok.com/search?q=thebeachwaver_reviews%20Smart%20WiFi%20COB%20Flexible%20Neon%20Rope%20LED%20Strip%20Light%2016.4ft%20Music%20Sync</t>
         </is>
       </c>
     </row>
@@ -14129,7 +14129,7 @@
       </c>
       <c r="L10" s="5" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@cleanwithme_asmr/video/7543817293019</t>
+          <t>https://www.tiktok.com/search?q=led_vibes_room%20Electric%20Spin%20Scrubber%20360%20Cordless%20Power%20Shower%20Cleaner%20Brush</t>
         </is>
       </c>
     </row>
@@ -14187,7 +14187,7 @@
       </c>
       <c r="L11" s="5" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@wavytalkofficial/video/744982736192</t>
+          <t>https://www.tiktok.com/search?q=cleanwithme_asmr_reviews%20Wavytalk%20Thermal%20Round%20Brush%201.5%20Inch%20Ceramic%20Heated%20Blowout%20Brush</t>
         </is>
       </c>
     </row>
@@ -14245,7 +14245,7 @@
       </c>
       <c r="L12" s="5" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@owala_official/video/7542817293019</t>
+          <t>https://www.tiktok.com/search?q=wavytalkofficial%20Owala%20FreeSip%2032oz%20Insulated%20Stainless%20Steel%20Water%20Bottle%20Tumbler</t>
         </is>
       </c>
     </row>
@@ -14303,7 +14303,7 @@
       </c>
       <c r="L13" s="5" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@urban_threads_men/video/7425982736192</t>
+          <t>https://www.tiktok.com/search?q=owala_official_reviews%20Baggy%20Parachute%20Cargo%20Streetwear%20Pants%20Multi-Pocket%20Tactical%20Fit</t>
         </is>
       </c>
     </row>
@@ -14361,7 +14361,7 @@
       </c>
       <c r="L14" s="5" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@personalized_glam/video/7422982736192</t>
+          <t>https://www.tiktok.com/search?q=urban_threads_men%20Custom%20Birth%20Flower%20Bar%20Name%20Pendant%20Necklace%2018K%20Gold%20Plated</t>
         </is>
       </c>
     </row>
@@ -14419,7 +14419,7 @@
       </c>
       <c r="L15" s="5" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@health_gurus_us/video/7419982736192</t>
+          <t>https://www.tiktok.com/search?q=personalized_glam%20Magnesium%20Glycinate%20Deep%20Sleep%20Relax%20Gummies%2060ct%20High%20Absorption</t>
         </is>
       </c>
     </row>
@@ -14477,7 +14477,7 @@
       </c>
       <c r="L16" s="5" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@halara_official/video/745982736192</t>
+          <t>https://www.tiktok.com/search?q=health_gurus_us%20Halara%20High%20Waisted%20Crossover%20Side%20Pocket%20Flared%20Casual%20Leggings</t>
         </is>
       </c>
     </row>
@@ -14535,7 +14535,7 @@
       </c>
       <c r="L17" s="5" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@cloud_cushion_slides/video/7428982736192</t>
+          <t>https://www.tiktok.com/search?q=halara_official%20Ultra-Thick%20Cloud%20Cushion%20Ergonomic%20Recovery%20Slides%20Anti-Slip</t>
         </is>
       </c>
     </row>
@@ -14593,7 +14593,7 @@
       </c>
       <c r="L18" s="5" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@keychron_official/video/7548817293019</t>
+          <t>https://www.tiktok.com/search?q=cloud_cushion_slides%20Wireless%20Custom%20Mechanical%20Keyboard%20RGB%20Hot-Swappable%20Gateron%20Pro</t>
         </is>
       </c>
     </row>
@@ -14651,7 +14651,7 @@
       </c>
       <c r="L19" s="5" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@ergonomic_living/video/7551817293019</t>
+          <t>https://www.tiktok.com/search?q=keychron_official_reviews%20Breathable%20Mesh%20Ergonomic%20Office%20Chair%20with%203D%20Lumbar%20Support</t>
         </is>
       </c>
     </row>
@@ -14709,7 +14709,7 @@
       </c>
       <c r="L20" s="5" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@vintage_vault_us/video/7427982736192</t>
+          <t>https://www.tiktok.com/search?q=ergonomic_living_reviews%20Authentic%2090s%20Carhartt%20Detroit%20Jacket%20Vintage%20Distressed%20Blanket%20Lined</t>
         </is>
       </c>
     </row>
@@ -14767,7 +14767,7 @@
       </c>
       <c r="L21" s="5" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@tartecosmetics/video/746982736192</t>
+          <t>https://www.tiktok.com/search?q=vintage_vault_us%20Tarte%20Maracuja%20Juicy%20Lip%20Plump%20Viral%20Hydrating%20Gloss</t>
         </is>
       </c>
     </row>
@@ -14825,7 +14825,7 @@
       </c>
       <c r="L22" s="5" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@brookemonk_/video/748982736192</t>
+          <t>https://www.tiktok.com/search?q=tartecosmetics%20Anker%20MagGo%20Qi2%20Ultra-Fast%20Magnetic%20Power%20Bank%2010000mAh</t>
         </is>
       </c>
     </row>
@@ -14883,7 +14883,7 @@
       </c>
       <c r="L23" s="5" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@led_vibes_room/video/7553817293019</t>
+          <t>https://www.tiktok.com/search?q=brookemonk_%20Smart%20WiFi%20COB%20Flexible%20Neon%20Rope%20LED%20Strip%20Light%2016.4ft%20Music%20Sync</t>
         </is>
       </c>
     </row>
@@ -14941,7 +14941,7 @@
       </c>
       <c r="L24" s="5" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@neatfreak_home/video/7421982736192</t>
+          <t>https://www.tiktok.com/search?q=led_vibes_room_reviews%20Foldable%20Handheld%20Garment%20Clothes%20Steamer%201000W%20Fast%20Heat</t>
         </is>
       </c>
     </row>
@@ -14999,7 +14999,7 @@
       </c>
       <c r="L25" s="5" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@everyday_carry_us/video/7424982736192</t>
+          <t>https://www.tiktok.com/search?q=neatfreak_home%20Everyday%20Everywhere%20Water-Resistant%20Crossbody%20Belt%20Bag%20Adjustable</t>
         </is>
       </c>
     </row>
@@ -15057,7 +15057,7 @@
       </c>
       <c r="L26" s="5" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@wavytalkofficial/video/7537817293019</t>
+          <t>https://www.tiktok.com/search?q=everyday_carry_us%20Wavytalk%20Thermal%20Round%20Brush%201.5%20Inch%20Ceramic%20Heated%20Blowout%20Brush</t>
         </is>
       </c>
     </row>
@@ -15115,7 +15115,7 @@
       </c>
       <c r="L27" s="5" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@gurunanda.official/video/742982736192</t>
+          <t>https://www.tiktok.com/search?q=wavytalkofficial_reviews%20GuruNanda%20Cocomint%20Coconut%20Pulling%20Oil%20with%20Tongue%20Scraper</t>
         </is>
       </c>
     </row>
@@ -15173,7 +15173,7 @@
       </c>
       <c r="L28" s="5" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@urban_threads_men/video/7558817293019</t>
+          <t>https://www.tiktok.com/search?q=gurunanda.official%20Baggy%20Parachute%20Cargo%20Streetwear%20Pants%20Multi-Pocket%20Tactical%20Fit</t>
         </is>
       </c>
     </row>
@@ -15231,7 +15231,7 @@
       </c>
       <c r="L29" s="5" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@personalized_glam/video/7555817293019</t>
+          <t>https://www.tiktok.com/search?q=urban_threads_men_reviews%20Custom%20Birth%20Flower%20Bar%20Name%20Pendant%20Necklace%2018K%20Gold%20Plated</t>
         </is>
       </c>
     </row>
@@ -15289,7 +15289,7 @@
       </c>
       <c r="L30" s="5" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@health_gurus_us/video/7552817293019</t>
+          <t>https://www.tiktok.com/search?q=personalized_glam_reviews%20Magnesium%20Glycinate%20Deep%20Sleep%20Relax%20Gummies%2060ct%20High%20Absorption</t>
         </is>
       </c>
     </row>
@@ -15347,7 +15347,7 @@
       </c>
       <c r="L31" s="5" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@tool_master_diy/video/7431982736192</t>
+          <t>https://www.tiktok.com/search?q=health_gurus_us_reviews%204V%20Cordless%20Electric%20Screwdriver%20Rechargeable%2036%20Bit%20Set%20Magnetic%20Head</t>
         </is>
       </c>
     </row>
@@ -15405,7 +15405,7 @@
       </c>
       <c r="L32" s="5" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@fanttik_official/video/7411982736192</t>
+          <t>https://www.tiktok.com/search?q=tool_master_diy%20Portable%20Cordless%20Smart%20Tire%20Inflator%20%26%20Digital%20Air%20Compressor%20150%20PSI</t>
         </is>
       </c>
     </row>
@@ -15463,7 +15463,7 @@
       </c>
       <c r="L33" s="5" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@cleanskinclub/video/743982736192</t>
+          <t>https://www.tiktok.com/search?q=fanttik_official%20Clean%20Skin%20Club%20Clean%20Towels%20XL%20100%25%20Biobased%20Disposable%20Face%20Towels</t>
         </is>
       </c>
     </row>
@@ -15521,7 +15521,7 @@
       </c>
       <c r="L34" s="5" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@halara_official/video/7538817293019</t>
+          <t>https://www.tiktok.com/search?q=cleanskinclub%20Halara%20High%20Waisted%20Crossover%20Side%20Pocket%20Flared%20Casual%20Leggings</t>
         </is>
       </c>
     </row>
@@ -15579,7 +15579,7 @@
       </c>
       <c r="L35" s="5" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@cloud_cushion_slides/video/7561817293019</t>
+          <t>https://www.tiktok.com/search?q=halara_official_reviews%20Ultra-Thick%20Cloud%20Cushion%20Ergonomic%20Recovery%20Slides%20Anti-Slip</t>
         </is>
       </c>
     </row>
@@ -15637,7 +15637,7 @@
       </c>
       <c r="L36" s="5" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@crunchycandylab/video/7417982736192</t>
+          <t>https://www.tiktok.com/search?q=cloud_cushion_slides_reviews%20Freeze%20Dried%20Rainbow%20Crunch%20Crunchy%20Candy%208oz%20Party%20Pack</t>
         </is>
       </c>
     </row>
@@ -15695,7 +15695,7 @@
       </c>
       <c r="L37" s="5" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@vintage_vault_us/video/7560817293019</t>
+          <t>https://www.tiktok.com/search?q=crunchycandylab%20Authentic%2090s%20Carhartt%20Detroit%20Jacket%20Vintage%20Distressed%20Blanket%20Lined</t>
         </is>
       </c>
     </row>
@@ -15753,7 +15753,7 @@
       </c>
       <c r="L38" s="5" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@tartecosmetics/video/7539817293019</t>
+          <t>https://www.tiktok.com/search?q=vintage_vault_us_reviews%20Tarte%20Maracuja%20Juicy%20Lip%20Plump%20Viral%20Hydrating%20Gloss</t>
         </is>
       </c>
     </row>
@@ -15811,7 +15811,7 @@
       </c>
       <c r="L39" s="5" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@brookemonk_/video/7541817293019</t>
+          <t>https://www.tiktok.com/search?q=tartecosmetics_reviews%20Anker%20MagGo%20Qi2%20Ultra-Fast%20Magnetic%20Power%20Bank%2010000mAh</t>
         </is>
       </c>
     </row>
@@ -15869,7 +15869,7 @@
       </c>
       <c r="L40" s="5" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@neatfreak_home/video/7554817293019</t>
+          <t>https://www.tiktok.com/search?q=brookemonk__reviews%20Foldable%20Handheld%20Garment%20Clothes%20Steamer%201000W%20Fast%20Heat</t>
         </is>
       </c>
     </row>
@@ -15927,7 +15927,7 @@
       </c>
       <c r="L41" s="5" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@everyday_carry_us/video/7557817293019</t>
+          <t>https://www.tiktok.com/search?q=neatfreak_home_reviews%20Everyday%20Everywhere%20Water-Resistant%20Crossbody%20Belt%20Bag%20Adjustable</t>
         </is>
       </c>
     </row>
@@ -15985,7 +15985,7 @@
       </c>
       <c r="L42" s="5" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@gurunanda.official/video/7535817293019</t>
+          <t>https://www.tiktok.com/search?q=everyday_carry_us_reviews%20GuruNanda%20Cocomint%20Coconut%20Pulling%20Oil%20with%20Tongue%20Scraper</t>
         </is>
       </c>
     </row>
@@ -16043,7 +16043,7 @@
       </c>
       <c r="L43" s="5" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@popflexactive/video/7429982736192</t>
+          <t>https://www.tiktok.com/search?q=gurunanda.official_reviews%20Wide%20Band%20Non-Slip%20Booty%20Fabric%20Resistance%20Bands%203pk%20Heavy%20Duty</t>
         </is>
       </c>
     </row>
@@ -16101,7 +16101,7 @@
       </c>
       <c r="L44" s="5" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@fanttik_official/video/7544817293019</t>
+          <t>https://www.tiktok.com/search?q=popflexactive%20Portable%20Cordless%20Smart%20Tire%20Inflator%20%26%20Digital%20Air%20Compressor%20150%20PSI</t>
         </is>
       </c>
     </row>
@@ -16159,7 +16159,7 @@
       </c>
       <c r="L45" s="5" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@cleanskinclub/video/7536817293019</t>
+          <t>https://www.tiktok.com/search?q=fanttik_official_reviews%20Clean%20Skin%20Club%20Clean%20Towels%20XL%20100%25%20Biobased%20Disposable%20Face%20Towels</t>
         </is>
       </c>
     </row>
@@ -16217,7 +16217,7 @@
       </c>
       <c r="L46" s="5" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@crunchycandylab/video/7550817293019</t>
+          <t>https://www.tiktok.com/search?q=cleanskinclub_reviews%20Freeze%20Dried%20Rainbow%20Crunch%20Crunchy%20Candy%208oz%20Party%20Pack</t>
         </is>
       </c>
     </row>
@@ -16275,7 +16275,7 @@
       </c>
       <c r="L47" s="5" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@y2k_retro_shades/video/7416982736192</t>
+          <t>https://www.tiktok.com/search?q=crunchycandylab_reviews%20Retro%20Oval%20Chunky%20Y2K%20Polarized%20UV400%20Sunglasses</t>
         </is>
       </c>
     </row>
@@ -16333,7 +16333,7 @@
       </c>
       <c r="L48" s="5" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@brodiethatdood/video/747982736192</t>
+          <t>https://www.tiktok.com/search?q=y2k_retro_shades%20Aumuca%20Self-Cleaning%20Slicker%20Deshedding%20Brush%20for%20Dogs%20and%20Cats</t>
         </is>
       </c>
     </row>
@@ -16391,7 +16391,7 @@
       </c>
       <c r="L49" s="5" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@tiny_trends_kids/video/7423982736192</t>
+          <t>https://www.tiktok.com/search?q=brodiethatdood%20Toddler%202-Piece%20Waffle%20Knit%20Loungewear%20Set%20Soft%20Organic%20Cotton</t>
         </is>
       </c>
     </row>
@@ -16449,7 +16449,7 @@
       </c>
       <c r="L50" s="5" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@card_collector_us/video/7414982736192</t>
+          <t>https://www.tiktok.com/search?q=tiny_trends_kids%20Pokemon%20PTCG%20Booster%20Binder%20%26%20Magnetic%20Acrylic%20Storage%20Cases</t>
         </is>
       </c>
     </row>
@@ -16507,7 +16507,7 @@
       </c>
       <c r="L51" s="5" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@digital_planner_club/video/7433982736192</t>
+          <t>https://www.tiktok.com/search?q=card_collector_us%20Ultimate%20Life%20OS%20All-in-One%20Notion%20Template%202026%20Daily%20Habit%20Tracker</t>
         </is>
       </c>
     </row>
@@ -16565,7 +16565,7 @@
       </c>
       <c r="L52" s="5" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@aesthetic_home_rugs/video/7430982736192</t>
+          <t>https://www.tiktok.com/search?q=digital_planner_club%20Super%20Absorbent%20Visual%20Memory%20Foam%20Floor%20Mat%20Instant%20Dry%20Bathroom%20Rug</t>
         </is>
       </c>
     </row>
@@ -16623,7 +16623,7 @@
       </c>
       <c r="L53" s="5" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@popflexactive/video/7562817293019</t>
+          <t>https://www.tiktok.com/search?q=aesthetic_home_rugs%20Wide%20Band%20Non-Slip%20Booty%20Fabric%20Resistance%20Bands%203pk%20Heavy%20Duty</t>
         </is>
       </c>
     </row>
@@ -16681,7 +16681,7 @@
       </c>
       <c r="L54" s="5" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@mommy_finds_daily/video/7412982736192</t>
+          <t>https://www.tiktok.com/search?q=popflexactive_reviews%20Silicone%20Pull%20String%20Sensory%20Montessori%20Teething%20Toy%20for%20Babies</t>
         </is>
       </c>
     </row>
@@ -16739,7 +16739,7 @@
       </c>
       <c r="L55" s="5" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@fidget_satisfying/video/7432982736192</t>
+          <t>https://www.tiktok.com/search?q=mommy_finds_daily%20Steamed%20Bun%20Dumpling%20Squishy%20Stress%20Relief%20Slow-Rise%20Sensory%20Toy</t>
         </is>
       </c>
     </row>
@@ -16797,7 +16797,7 @@
       </c>
       <c r="L56" s="5" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@modest_chic_us/video/7426982736192</t>
+          <t>https://www.tiktok.com/search?q=fidget_satisfying%20Premium%20Modal%20Cotton%20Jersey%20Breathable%20Instant%20Hijab%20Scarf</t>
         </is>
       </c>
     </row>
@@ -16855,7 +16855,7 @@
       </c>
       <c r="L57" s="5" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@y2k_retro_shades/video/7549817293019</t>
+          <t>https://www.tiktok.com/search?q=modest_chic_us%20Retro%20Oval%20Chunky%20Y2K%20Polarized%20UV400%20Sunglasses</t>
         </is>
       </c>
     </row>
@@ -16913,7 +16913,7 @@
       </c>
       <c r="L58" s="5" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@brodiethatdood/video/7540817293019</t>
+          <t>https://www.tiktok.com/search?q=y2k_retro_shades_reviews%20Aumuca%20Self-Cleaning%20Slicker%20Deshedding%20Brush%20for%20Dogs%20and%20Cats</t>
         </is>
       </c>
     </row>
@@ -16971,7 +16971,7 @@
       </c>
       <c r="L59" s="5" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@tiny_trends_kids/video/7556817293019</t>
+          <t>https://www.tiktok.com/search?q=brodiethatdood_reviews%20Toddler%202-Piece%20Waffle%20Knit%20Loungewear%20Set%20Soft%20Organic%20Cotton</t>
         </is>
       </c>
     </row>
@@ -17029,7 +17029,7 @@
       </c>
       <c r="L60" s="5" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@card_collector_us/video/7547817293019</t>
+          <t>https://www.tiktok.com/search?q=tiny_trends_kids_reviews%20Pokemon%20PTCG%20Booster%20Binder%20%26%20Magnetic%20Acrylic%20Storage%20Cases</t>
         </is>
       </c>
     </row>
@@ -17087,7 +17087,7 @@
       </c>
       <c r="L61" s="5" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@journaling_aesthetic/video/7413982736192</t>
+          <t>https://www.tiktok.com/search?q=card_collector_us_reviews%20Vintage%20Embossed%20Hardcover%20Lock%20Journal%20%26%20Planner%20with%20Metal%20Clasp</t>
         </is>
       </c>
     </row>
@@ -17145,7 +17145,7 @@
       </c>
       <c r="L62" s="5" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@mommy_finds_daily/video/7545817293019</t>
+          <t>https://www.tiktok.com/search?q=journaling_aesthetic%20Silicone%20Pull%20String%20Sensory%20Montessori%20Teething%20Toy%20for%20Babies</t>
         </is>
       </c>
     </row>
@@ -17203,7 +17203,7 @@
       </c>
       <c r="L63" s="5" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@modest_chic_us/video/7559817293019</t>
+          <t>https://www.tiktok.com/search?q=mommy_finds_daily_reviews%20Premium%20Modal%20Cotton%20Jersey%20Breathable%20Instant%20Hijab%20Scarf</t>
         </is>
       </c>
     </row>
@@ -17261,7 +17261,7 @@
       </c>
       <c r="L64" s="5" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@journaling_aesthetic/video/7546817293019</t>
+          <t>https://www.tiktok.com/search?q=modest_chic_us_reviews%20Vintage%20Embossed%20Hardcover%20Lock%20Journal%20%26%20Planner%20with%20Metal%20Clasp</t>
         </is>
       </c>
     </row>
@@ -17532,17 +17532,17 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>owala_official</t>
+          <t>Owala’s life</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>@owala_official</t>
+          <t>@owalalife</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>1.2M</t>
+          <t>1.0K</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
@@ -17570,12 +17570,12 @@
       </c>
       <c r="J5" s="3" t="inlineStr">
         <is>
-          <t>10.2%</t>
+          <t>8.5%</t>
         </is>
       </c>
       <c r="K5" s="5" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@owala_official</t>
+          <t>https://www.tiktok.com/@owalalife</t>
         </is>
       </c>
     </row>
@@ -17744,12 +17744,12 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>keychron_official</t>
+          <t>keychron</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>@keychron_official</t>
+          <t>@keychron</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
@@ -17787,7 +17787,7 @@
       </c>
       <c r="K9" s="5" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@keychron_official</t>
+          <t>https://www.tiktok.com/@keychron</t>
         </is>
       </c>
     </row>

</xml_diff>